<commit_message>
Remove the retired client catalog row from the feature ledger
Drops PF-PROJ-015 from output/spreadsheet/portfolio-feature-ledger.xlsx so
the workbook no longer references the removed project or its domain. Other
Feature IDs stay stable; Summary counts, formulas, and the autofilter range
follow the 77 remaining stories, and rule 7 records the removal.

Co-authored-by: Steve Defendre <Sdefendre@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/spreadsheet/portfolio-feature-ledger.xlsx
+++ b/output/spreadsheet/portfolio-feature-ledger.xlsx
@@ -24,7 +24,7 @@
     <definedName name="VerificationStatuses">'Lists'!$F$2:$F$6</definedName>
     <definedName name="FixStatuses">'Lists'!$J$2:$J$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Summary'!$A$1:$F$40</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Features'!$A$1:$V$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Features'!$A$1:$V$78</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Features'!$1:$1,'Features'!$A:$D</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Features'!$A$1:$V$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Defects'!$A$1:$R$14</definedName>
@@ -629,7 +629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -650,10 +650,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Canonical 78-story post-fix reconciliation — 2026-08-23 14:31 America/New_York</t>
-        </is>
-      </c>
-    </row>
+          <t>Canonical 77-story post-fix reconciliation — 2026-08-23 14:31 America/New_York</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -680,7 +681,7 @@
     </row>
     <row r="6">
       <c r="A6" s="5">
-        <f>COUNTA(Features!$A$2:$A$79)</f>
+        <f>COUNTA(Features!$A$2:$A$78)</f>
         <v/>
       </c>
       <c r="C6" s="5">
@@ -692,6 +693,7 @@
         <v/>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -733,7 +735,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIF(Features!$B$2:$B$79,A10)</f>
+        <f>COUNTIF(Features!$B$2:$B$78,A10)</f>
         <v/>
       </c>
       <c r="C10">
@@ -756,7 +758,7 @@
         </is>
       </c>
       <c r="B11">
-        <f>COUNTIF(Features!$B$2:$B$79,A11)</f>
+        <f>COUNTIF(Features!$B$2:$B$78,A11)</f>
         <v/>
       </c>
       <c r="C11">
@@ -779,7 +781,7 @@
         </is>
       </c>
       <c r="B12">
-        <f>COUNTIF(Features!$B$2:$B$79,A12)</f>
+        <f>COUNTIF(Features!$B$2:$B$78,A12)</f>
         <v/>
       </c>
       <c r="C12">
@@ -802,7 +804,7 @@
         </is>
       </c>
       <c r="B13">
-        <f>COUNTIF(Features!$B$2:$B$79,A13)</f>
+        <f>COUNTIF(Features!$B$2:$B$78,A13)</f>
         <v/>
       </c>
       <c r="C13">
@@ -825,7 +827,7 @@
         </is>
       </c>
       <c r="B14">
-        <f>COUNTIF(Features!$B$2:$B$79,A14)</f>
+        <f>COUNTIF(Features!$B$2:$B$78,A14)</f>
         <v/>
       </c>
       <c r="C14">
@@ -897,7 +899,7 @@
         </is>
       </c>
       <c r="B17">
-        <f>COUNTIF(Features!$M$2:$M$79,A17)</f>
+        <f>COUNTIF(Features!$M$2:$M$78,A17)</f>
         <v/>
       </c>
       <c r="C17" t="inlineStr">
@@ -906,7 +908,7 @@
         </is>
       </c>
       <c r="D17">
-        <f>COUNTIF(Features!$P$2:$P$79,C17)</f>
+        <f>COUNTIF(Features!$P$2:$P$78,C17)</f>
         <v/>
       </c>
       <c r="E17" t="inlineStr">
@@ -915,7 +917,7 @@
         </is>
       </c>
       <c r="F17">
-        <f>COUNTIF(Features!$Q$2:$Q$79,E17)</f>
+        <f>COUNTIF(Features!$Q$2:$Q$78,E17)</f>
         <v/>
       </c>
     </row>
@@ -926,7 +928,7 @@
         </is>
       </c>
       <c r="B18">
-        <f>COUNTIF(Features!$M$2:$M$79,A18)</f>
+        <f>COUNTIF(Features!$M$2:$M$78,A18)</f>
         <v/>
       </c>
       <c r="C18" t="inlineStr">
@@ -935,7 +937,7 @@
         </is>
       </c>
       <c r="D18">
-        <f>COUNTIF(Features!$P$2:$P$79,C18)</f>
+        <f>COUNTIF(Features!$P$2:$P$78,C18)</f>
         <v/>
       </c>
       <c r="E18" t="inlineStr">
@@ -944,7 +946,7 @@
         </is>
       </c>
       <c r="F18">
-        <f>COUNTIF(Features!$Q$2:$Q$79,E18)</f>
+        <f>COUNTIF(Features!$Q$2:$Q$78,E18)</f>
         <v/>
       </c>
     </row>
@@ -955,7 +957,7 @@
         </is>
       </c>
       <c r="B19">
-        <f>COUNTIF(Features!$M$2:$M$79,A19)</f>
+        <f>COUNTIF(Features!$M$2:$M$78,A19)</f>
         <v/>
       </c>
       <c r="C19" t="inlineStr">
@@ -964,7 +966,7 @@
         </is>
       </c>
       <c r="D19">
-        <f>COUNTIF(Features!$P$2:$P$79,C19)</f>
+        <f>COUNTIF(Features!$P$2:$P$78,C19)</f>
         <v/>
       </c>
       <c r="E19" t="inlineStr">
@@ -973,7 +975,7 @@
         </is>
       </c>
       <c r="F19">
-        <f>COUNTIF(Features!$Q$2:$Q$79,E19)</f>
+        <f>COUNTIF(Features!$Q$2:$Q$78,E19)</f>
         <v/>
       </c>
     </row>
@@ -984,7 +986,7 @@
         </is>
       </c>
       <c r="B20">
-        <f>COUNTIF(Features!$M$2:$M$79,A20)</f>
+        <f>COUNTIF(Features!$M$2:$M$78,A20)</f>
         <v/>
       </c>
       <c r="C20" t="inlineStr">
@@ -993,7 +995,7 @@
         </is>
       </c>
       <c r="D20">
-        <f>COUNTIF(Features!$P$2:$P$79,C20)</f>
+        <f>COUNTIF(Features!$P$2:$P$78,C20)</f>
         <v/>
       </c>
       <c r="E20" t="inlineStr">
@@ -1002,7 +1004,7 @@
         </is>
       </c>
       <c r="F20">
-        <f>COUNTIF(Features!$Q$2:$Q$79,E20)</f>
+        <f>COUNTIF(Features!$Q$2:$Q$78,E20)</f>
         <v/>
       </c>
     </row>
@@ -1013,7 +1015,7 @@
         </is>
       </c>
       <c r="B21">
-        <f>COUNTIF(Features!$M$2:$M$79,A21)</f>
+        <f>COUNTIF(Features!$M$2:$M$78,A21)</f>
         <v/>
       </c>
       <c r="C21" t="inlineStr">
@@ -1022,7 +1024,7 @@
         </is>
       </c>
       <c r="D21">
-        <f>COUNTIF(Features!$P$2:$P$79,C21)</f>
+        <f>COUNTIF(Features!$P$2:$P$78,C21)</f>
         <v/>
       </c>
       <c r="E21" t="inlineStr">
@@ -1031,10 +1033,12 @@
         </is>
       </c>
       <c r="F21">
-        <f>COUNTIF(Features!$Q$2:$Q$79,E21)</f>
+        <f>COUNTIF(Features!$Q$2:$Q$78,E21)</f>
         <v/>
       </c>
     </row>
+    <row r="22"/>
+    <row r="23"/>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
@@ -1242,6 +1246,7 @@
         <v/>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
@@ -1252,7 +1257,7 @@
     <row r="35" ht="38" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>1. All 78 stories retain canonical baseline status/evidence and now have a final Post-Fix Status of Pass or Blocked; Post-Fix Fail and Not Run are zero.</t>
+          <t>1. All 77 stories retain canonical baseline status/evidence and now have a final Post-Fix Status of Pass or Blocked; Post-Fix Fail and Not Run are zero.</t>
         </is>
       </c>
       <c r="B35" s="19" t="n"/>
@@ -1321,11 +1326,24 @@
       <c r="E40" s="19" t="n"/>
       <c r="F40" s="19" t="n"/>
     </row>
+    <row r="41" ht="38" customHeight="1">
+      <c r="A41" s="21" t="inlineStr">
+        <is>
+          <t>7. PF-PROJ-015, the catalog story for a client project that left the portfolio, was removed on 2026-10-13; the remaining Feature IDs are unchanged.</t>
+        </is>
+      </c>
+      <c r="B41" s="19" t="n"/>
+      <c r="C41" s="19" t="n"/>
+      <c r="D41" s="19" t="n"/>
+      <c r="E41" s="19" t="n"/>
+      <c r="F41" s="19" t="n"/>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="16">
+  <mergeCells count="17">
     <mergeCell ref="A38:F38"/>
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A41:F41"/>
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A36:F36"/>
@@ -1361,7 +1379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V79"/>
+  <dimension ref="A1:V78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5795,7 +5813,7 @@
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>PF-PROJ-015</t>
+          <t>PF-PROJ-016</t>
         </is>
       </c>
       <c r="B44" s="13" t="inlineStr">
@@ -5805,7 +5823,7 @@
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>Project catalog: Krystin Sylvia</t>
+          <t>Project catalog: Velocity Care LLC</t>
         </is>
       </c>
       <c r="D44" s="13" t="inlineStr">
@@ -5815,7 +5833,7 @@
       </c>
       <c r="E44" s="13" t="inlineStr">
         <is>
-          <t>As a visitor, I want healthcare portfolio proof.</t>
+          <t>As a visitor, I want healthcare-practice proof.</t>
         </is>
       </c>
       <c r="F44" s="13" t="inlineStr">
@@ -5825,12 +5843,12 @@
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>Open “View portfolio.”</t>
+          <t>Open “Visit healthcare site.”</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr">
         <is>
-          <t>Show 2026 Live client details and open https://krystinsylvia.com.</t>
+          <t>Show 2026 Live client details and open https://velocitycarellc.com.</t>
         </is>
       </c>
       <c r="I44" s="13" t="inlineStr">
@@ -5840,7 +5858,7 @@
       </c>
       <c r="J44" s="13" t="inlineStr">
         <is>
-          <t>src/data/projects.ts:61-69</t>
+          <t>src/data/projects.ts:70-78</t>
         </is>
       </c>
       <c r="K44" s="13" t="inlineStr">
@@ -5860,7 +5878,7 @@
       </c>
       <c r="N44" s="13" t="inlineStr">
         <is>
-          <t>Pass — All expected content and https://www.krystinsylvia.com/ destination were present. Evidence: /tmp/portfolio-feature-audit/baseline/projects/interaction-evidence.md; /tmp/portfolio-feature-audit/baseline/projects/1440/projects-all-full.png</t>
+          <t>Pass — All expected content and https://www.velocitycarellc.com/ destination were present. Evidence: /tmp/portfolio-feature-audit/baseline/projects/interaction-evidence.md; /tmp/portfolio-feature-audit/baseline/projects/1440/projects-all-full.png</t>
         </is>
       </c>
       <c r="O44" s="13" t="n"/>
@@ -5876,7 +5894,7 @@
       </c>
       <c r="R44" s="13" t="inlineStr">
         <is>
-          <t>Pass — Catalog details, complete case study, CTA/new-tab name, and https://www.krystinsylvia.com/ destination matched. Evidence: /tmp/portfolio-feature-audit/postfix/projects/catalog-audit.json</t>
+          <t>Pass — Catalog details, complete case study, CTA/new-tab name, and https://www.velocitycarellc.com/ destination matched. Evidence: /tmp/portfolio-feature-audit/postfix/projects/catalog-audit.json</t>
         </is>
       </c>
       <c r="S44" s="13" t="inlineStr"/>
@@ -5895,7 +5913,7 @@
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>PF-PROJ-016</t>
+          <t>PF-PROJ-017</t>
         </is>
       </c>
       <c r="B45" s="13" t="inlineStr">
@@ -5905,7 +5923,7 @@
       </c>
       <c r="C45" s="13" t="inlineStr">
         <is>
-          <t>Project catalog: Velocity Care LLC</t>
+          <t>Project catalog: Command.AI</t>
         </is>
       </c>
       <c r="D45" s="13" t="inlineStr">
@@ -5915,22 +5933,22 @@
       </c>
       <c r="E45" s="13" t="inlineStr">
         <is>
-          <t>As a visitor, I want healthcare-practice proof.</t>
+          <t>As a visitor, I want veteran-platform product proof.</t>
         </is>
       </c>
       <c r="F45" s="13" t="inlineStr">
         <is>
-          <t>All/Client visible.</t>
+          <t>All/Product visible.</t>
         </is>
       </c>
       <c r="G45" s="13" t="inlineStr">
         <is>
-          <t>Open “Visit healthcare site.”</t>
+          <t>Open “Open platform.”</t>
         </is>
       </c>
       <c r="H45" s="13" t="inlineStr">
         <is>
-          <t>Show 2026 Live client details and open https://velocitycarellc.com.</t>
+          <t>Show 2026 Live product details and open https://trycommand.vercel.app.</t>
         </is>
       </c>
       <c r="I45" s="13" t="inlineStr">
@@ -5940,12 +5958,12 @@
       </c>
       <c r="J45" s="13" t="inlineStr">
         <is>
-          <t>src/data/projects.ts:70-78</t>
+          <t>src/data/projects.ts:79-87</t>
         </is>
       </c>
       <c r="K45" s="13" t="inlineStr">
         <is>
-          <t>src/data/__tests__/projects.test.ts:14-134; client-count E2E e2e/projects.spec.ts:11-15</t>
+          <t>src/data/__tests__/projects.test.ts:14-134</t>
         </is>
       </c>
       <c r="L45" s="13" t="inlineStr">
@@ -5960,7 +5978,7 @@
       </c>
       <c r="N45" s="13" t="inlineStr">
         <is>
-          <t>Pass — All expected content and https://www.velocitycarellc.com/ destination were present. Evidence: /tmp/portfolio-feature-audit/baseline/projects/interaction-evidence.md; /tmp/portfolio-feature-audit/baseline/projects/1440/projects-all-full.png</t>
+          <t>Pass — All expected content and https://trycommand.vercel.app/ destination were present. Evidence: /tmp/portfolio-feature-audit/baseline/projects/interaction-evidence.md; /tmp/portfolio-feature-audit/baseline/projects/1440/projects-all-full.png</t>
         </is>
       </c>
       <c r="O45" s="13" t="n"/>
@@ -5976,7 +5994,7 @@
       </c>
       <c r="R45" s="13" t="inlineStr">
         <is>
-          <t>Pass — Catalog details, complete case study, CTA/new-tab name, and https://www.velocitycarellc.com/ destination matched. Evidence: /tmp/portfolio-feature-audit/postfix/projects/catalog-audit.json</t>
+          <t>Pass — Catalog details, complete case study, CTA/new-tab name, and https://trycommand.vercel.app/ destination matched and opened in a new tab. Evidence: /tmp/portfolio-feature-audit/postfix/projects/catalog-audit.json; /tmp/portfolio-feature-audit/postfix/projects/interaction-evidence.md</t>
         </is>
       </c>
       <c r="S45" s="13" t="inlineStr"/>
@@ -5995,7 +6013,7 @@
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>PF-PROJ-017</t>
+          <t>PF-CONTACT-001</t>
         </is>
       </c>
       <c r="B46" s="13" t="inlineStr">
@@ -6005,47 +6023,47 @@
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>Project catalog: Command.AI</t>
+          <t>/contact route metadata</t>
         </is>
       </c>
       <c r="D46" s="13" t="inlineStr">
         <is>
-          <t>Visitor</t>
+          <t>Search/social crawler</t>
         </is>
       </c>
       <c r="E46" s="13" t="inlineStr">
         <is>
-          <t>As a visitor, I want veteran-platform product proof.</t>
+          <t>As a crawler, I want project-inquiry metadata.</t>
         </is>
       </c>
       <c r="F46" s="13" t="inlineStr">
         <is>
-          <t>All/Product visible.</t>
+          <t>Contact route requested.</t>
         </is>
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>Open “Open platform.”</t>
+          <t>Parse metadata.</t>
         </is>
       </c>
       <c r="H46" s="13" t="inlineStr">
         <is>
-          <t>Show 2026 Live product details and open https://trycommand.vercel.app.</t>
+          <t>Use Contact title/description, canonical /contact, and matching Open Graph URL/content.</t>
         </is>
       </c>
       <c r="I46" s="13" t="inlineStr">
         <is>
-          <t>Common card/accessibility rules apply.</t>
+          <t>No visual behavior.</t>
         </is>
       </c>
       <c r="J46" s="13" t="inlineStr">
         <is>
-          <t>src/data/projects.ts:79-87</t>
+          <t>src/app/(site)/contact/page.tsx:11-24</t>
         </is>
       </c>
       <c r="K46" s="13" t="inlineStr">
         <is>
-          <t>src/data/__tests__/projects.test.ts:14-134</t>
+          <t>src/app/(site)/contact/page.test.tsx:60-66</t>
         </is>
       </c>
       <c r="L46" s="13" t="inlineStr">
@@ -6060,13 +6078,17 @@
       </c>
       <c r="N46" s="13" t="inlineStr">
         <is>
-          <t>Pass — All expected content and https://trycommand.vercel.app/ destination were present. Evidence: /tmp/portfolio-feature-audit/baseline/projects/interaction-evidence.md; /tmp/portfolio-feature-audit/baseline/projects/1440/projects-all-full.png</t>
-        </is>
-      </c>
-      <c r="O46" s="13" t="n"/>
+          <t>Pass — Content/path matched locally and public canonical/OG consistently used the production origin. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md; /tmp/portfolio-feature-audit/baseline/contact-system/390/contact-full.png</t>
+        </is>
+      </c>
+      <c r="O46" s="13" t="inlineStr">
+        <is>
+          <t>CAND-RUNTIME-METADATA-001</t>
+        </is>
+      </c>
       <c r="P46" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Won't Fix</t>
         </is>
       </c>
       <c r="Q46" s="13" t="inlineStr">
@@ -6076,7 +6098,7 @@
       </c>
       <c r="R46" s="13" t="inlineStr">
         <is>
-          <t>Pass — Catalog details, complete case study, CTA/new-tab name, and https://trycommand.vercel.app/ destination matched and opened in a new tab. Evidence: /tmp/portfolio-feature-audit/postfix/projects/catalog-audit.json; /tmp/portfolio-feature-audit/postfix/projects/interaction-evidence.md</t>
+          <t>Pass — Contact returned 200 with route-specific title, description, canonical path, Open Graph URL, and expected content; local absolute URLs use the documented no-env localhost fallback. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-initial.png; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
         </is>
       </c>
       <c r="S46" s="13" t="inlineStr"/>
@@ -6095,7 +6117,7 @@
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>PF-CONTACT-001</t>
+          <t>PF-CONTACT-002</t>
         </is>
       </c>
       <c r="B47" s="13" t="inlineStr">
@@ -6105,47 +6127,47 @@
       </c>
       <c r="C47" s="13" t="inlineStr">
         <is>
-          <t>/contact route metadata</t>
+          <t>/contact primary inquiry</t>
         </is>
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>Search/social crawler</t>
+          <t>Prospect</t>
         </is>
       </c>
       <c r="E47" s="13" t="inlineStr">
         <is>
-          <t>As a crawler, I want project-inquiry metadata.</t>
+          <t>As a prospect, I want Steve’s direct email and availability.</t>
         </is>
       </c>
       <c r="F47" s="13" t="inlineStr">
         <is>
-          <t>Contact route requested.</t>
+          <t>Primary contact record exists.</t>
         </is>
       </c>
       <c r="G47" s="13" t="inlineStr">
         <is>
-          <t>Parse metadata.</t>
+          <t>Read primary contact panel.</t>
         </is>
       </c>
       <c r="H47" s="13" t="inlineStr">
         <is>
-          <t>Use Contact title/description, canonical /contact, and matching Open Graph URL/content.</t>
+          <t>Show availability, email address, description, direct email CTA, and copy control.</t>
         </is>
       </c>
       <c r="I47" s="13" t="inlineStr">
         <is>
-          <t>No visual behavior.</t>
+          <t>Large email wraps/breaks on mobile; labelled section; CTA stack switches to row at sm.</t>
         </is>
       </c>
       <c r="J47" s="13" t="inlineStr">
         <is>
-          <t>src/app/(site)/contact/page.tsx:11-24</t>
+          <t>src/app/(site)/contact/page.tsx:26-41,43-102; src/data/socials.ts:31-39</t>
         </is>
       </c>
       <c r="K47" s="13" t="inlineStr">
         <is>
-          <t>src/app/(site)/contact/page.test.tsx:60-66</t>
+          <t>src/app/(site)/contact/page.test.tsx:5-26; e2e/contact.spec.ts:31-44</t>
         </is>
       </c>
       <c r="L47" s="13" t="inlineStr">
@@ -6160,12 +6182,12 @@
       </c>
       <c r="N47" s="13" t="inlineStr">
         <is>
-          <t>Pass — Content/path matched locally and public canonical/OG consistently used the production origin. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md; /tmp/portfolio-feature-audit/baseline/contact-system/390/contact-full.png</t>
+          <t>Pass — All content and controls rendered; email wrapped without overflow and CTA stack adapted by breakpoint. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/1440/contact-full.png; /tmp/portfolio-feature-audit/baseline/contact-system/390/contact-full.png</t>
         </is>
       </c>
       <c r="O47" s="13" t="inlineStr">
         <is>
-          <t>CAND-RUNTIME-METADATA-001</t>
+          <t>DESIGN-AI-001</t>
         </is>
       </c>
       <c r="P47" s="13" t="inlineStr">
@@ -6180,7 +6202,7 @@
       </c>
       <c r="R47" s="13" t="inlineStr">
         <is>
-          <t>Pass — Contact returned 200 with route-specific title, description, canonical path, Open Graph URL, and expected content; local absolute URLs use the documented no-env localhost fallback. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-initial.png; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
+          <t>Pass — Primary inquiry, email, availability, direct CTA, and copy control rendered at 390, 768, and 1440 with no horizontal overflow and responsive CTA layout. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-initial.png; /tmp/portfolio-feature-audit/postfix/contact-system/contact-768.png; /tmp/portfolio-feature-audit/postfix/contact-system/contact-1440-validation-copy-repeat.png</t>
         </is>
       </c>
       <c r="S47" s="13" t="inlineStr"/>
@@ -6199,7 +6221,7 @@
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>PF-CONTACT-002</t>
+          <t>PF-CONTACT-003</t>
         </is>
       </c>
       <c r="B48" s="13" t="inlineStr">
@@ -6209,7 +6231,7 @@
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>/contact primary inquiry</t>
+          <t>/contact direct mailto</t>
         </is>
       </c>
       <c r="D48" s="13" t="inlineStr">
@@ -6219,37 +6241,37 @@
       </c>
       <c r="E48" s="13" t="inlineStr">
         <is>
-          <t>As a prospect, I want Steve’s direct email and availability.</t>
+          <t>As a prospect, I want to open a blank email to Steve.</t>
         </is>
       </c>
       <c r="F48" s="13" t="inlineStr">
         <is>
-          <t>Primary contact record exists.</t>
+          <t>Mail client handles mailto:.</t>
         </is>
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>Read primary contact panel.</t>
+          <t>Activate “Email Steve.”</t>
         </is>
       </c>
       <c r="H48" s="13" t="inlineStr">
         <is>
-          <t>Show availability, email address, description, direct email CTA, and copy control.</t>
+          <t>Open mailto:steve@defendresolutions.com.</t>
         </is>
       </c>
       <c r="I48" s="13" t="inlineStr">
         <is>
-          <t>Large email wraps/breaks on mobile; labelled section; CTA stack switches to row at sm.</t>
+          <t>48px focusable CTA; safe-href validation.</t>
         </is>
       </c>
       <c r="J48" s="13" t="inlineStr">
         <is>
-          <t>src/app/(site)/contact/page.tsx:26-41,43-102; src/data/socials.ts:31-39</t>
+          <t>src/app/(site)/contact/page.tsx:91-100; src/data/socials.ts:31-39</t>
         </is>
       </c>
       <c r="K48" s="13" t="inlineStr">
         <is>
-          <t>src/app/(site)/contact/page.test.tsx:5-26; e2e/contact.spec.ts:31-44</t>
+          <t>src/app/(site)/contact/page.test.tsx:5-26</t>
         </is>
       </c>
       <c r="L48" s="13" t="inlineStr">
@@ -6264,17 +6286,13 @@
       </c>
       <c r="N48" s="13" t="inlineStr">
         <is>
-          <t>Pass — All content and controls rendered; email wrapped without overflow and CTA stack adapted by breakpoint. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/1440/contact-full.png; /tmp/portfolio-feature-audit/baseline/contact-system/390/contact-full.png</t>
-        </is>
-      </c>
-      <c r="O48" s="13" t="inlineStr">
-        <is>
-          <t>DESIGN-AI-001</t>
-        </is>
-      </c>
+          <t>Pass — Href and 48px geometry matched; handler launch was intentionally not invoked. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md; /tmp/portfolio-feature-audit/baseline/contact-system/snapshot-contact-390.txt</t>
+        </is>
+      </c>
+      <c r="O48" s="13" t="n"/>
       <c r="P48" s="13" t="inlineStr">
         <is>
-          <t>Won't Fix</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="Q48" s="13" t="inlineStr">
@@ -6284,7 +6302,7 @@
       </c>
       <c r="R48" s="13" t="inlineStr">
         <is>
-          <t>Pass — Primary inquiry, email, availability, direct CTA, and copy control rendered at 390, 768, and 1440 with no horizontal overflow and responsive CTA layout. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-initial.png; /tmp/portfolio-feature-audit/postfix/contact-system/contact-768.png; /tmp/portfolio-feature-audit/postfix/contact-system/contact-1440-validation-copy-repeat.png</t>
+          <t>Pass — Email Steve retained mailto:steve@defendresolutions.com and a 48px desktop target; no real mail client was launched. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/lane-c-trace.zip</t>
         </is>
       </c>
       <c r="S48" s="13" t="inlineStr"/>
@@ -6303,7 +6321,7 @@
     <row r="49">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>PF-CONTACT-003</t>
+          <t>PF-CONTACT-004</t>
         </is>
       </c>
       <c r="B49" s="13" t="inlineStr">
@@ -6313,47 +6331,47 @@
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>/contact direct mailto</t>
+          <t>/contact clipboard success</t>
         </is>
       </c>
       <c r="D49" s="13" t="inlineStr">
         <is>
-          <t>Prospect</t>
+          <t>Visitor</t>
         </is>
       </c>
       <c r="E49" s="13" t="inlineStr">
         <is>
-          <t>As a prospect, I want to open a blank email to Steve.</t>
+          <t>As a visitor, I want to copy Steve’s email.</t>
         </is>
       </c>
       <c r="F49" s="13" t="inlineStr">
         <is>
-          <t>Mail client handles mailto:.</t>
+          <t>Clipboard API available and permission granted.</t>
         </is>
       </c>
       <c r="G49" s="13" t="inlineStr">
         <is>
-          <t>Activate “Email Steve.”</t>
+          <t>Activate “Copy email.”</t>
         </is>
       </c>
       <c r="H49" s="13" t="inlineStr">
         <is>
-          <t>Open mailto:steve@defendresolutions.com.</t>
+          <t>Write email; button becomes “Copied”; polite status announces full address; reset to idle after 2.5s.</t>
         </is>
       </c>
       <c r="I49" s="13" t="inlineStr">
         <is>
-          <t>48px focusable CTA; safe-href validation.</t>
+          <t>Accessible status association via aria-describedby; icons decorative.</t>
         </is>
       </c>
       <c r="J49" s="13" t="inlineStr">
         <is>
-          <t>src/app/(site)/contact/page.tsx:91-100; src/data/socials.ts:31-39</t>
+          <t>src/components/CopyEmailButton.tsx:15-45,47-84</t>
         </is>
       </c>
       <c r="K49" s="13" t="inlineStr">
         <is>
-          <t>src/app/(site)/contact/page.test.tsx:5-26</t>
+          <t>src/components/__tests__/CopyEmailButton.test.tsx:29-46; e2e/contact.spec.ts:31-44</t>
         </is>
       </c>
       <c r="L49" s="13" t="inlineStr">
@@ -6368,7 +6386,7 @@
       </c>
       <c r="N49" s="13" t="inlineStr">
         <is>
-          <t>Pass — Href and 48px geometry matched; handler launch was intentionally not invoked. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md; /tmp/portfolio-feature-audit/baseline/contact-system/snapshot-contact-390.txt</t>
+          <t>Pass — Controlled clipboard success wrote the exact address, showed Copied/full polite status, then reset after 2.7s. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/interactions/copy-success.png; /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md</t>
         </is>
       </c>
       <c r="O49" s="13" t="n"/>
@@ -6384,7 +6402,7 @@
       </c>
       <c r="R49" s="13" t="inlineStr">
         <is>
-          <t>Pass — Email Steve retained mailto:steve@defendresolutions.com and a 48px desktop target; no real mail client was launched. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/lane-c-trace.zip</t>
+          <t>Pass — Controlled clipboard success wrote the exact address, announced success, changed the button to Copied, and reset after 2.6 seconds; exact-768 success also passed. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-copy-success.png; /tmp/portfolio-feature-audit/postfix/contact-system/lane-c-trace.zip</t>
         </is>
       </c>
       <c r="S49" s="13" t="inlineStr"/>
@@ -6403,7 +6421,7 @@
     <row r="50">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>PF-CONTACT-004</t>
+          <t>PF-CONTACT-005</t>
         </is>
       </c>
       <c r="B50" s="13" t="inlineStr">
@@ -6413,7 +6431,7 @@
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>/contact clipboard success</t>
+          <t>/contact clipboard failure</t>
         </is>
       </c>
       <c r="D50" s="13" t="inlineStr">
@@ -6423,37 +6441,37 @@
       </c>
       <c r="E50" s="13" t="inlineStr">
         <is>
-          <t>As a visitor, I want to copy Steve’s email.</t>
+          <t>As a visitor, I want recoverable feedback if copy fails.</t>
         </is>
       </c>
       <c r="F50" s="13" t="inlineStr">
         <is>
-          <t>Clipboard API available and permission granted.</t>
+          <t>Clipboard API missing/rejects.</t>
         </is>
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>Activate “Copy email.”</t>
+          <t>Activate copy.</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr">
         <is>
-          <t>Write email; button becomes “Copied”; polite status announces full address; reset to idle after 2.5s.</t>
+          <t>Button becomes “Try copy again” and status advises manual selection; no alert dialog.</t>
         </is>
       </c>
       <c r="I50" s="13" t="inlineStr">
         <is>
-          <t>Accessible status association via aria-describedby; icons decorative.</t>
+          <t>Polite live status; amber icon plus text.</t>
         </is>
       </c>
       <c r="J50" s="13" t="inlineStr">
         <is>
-          <t>src/components/CopyEmailButton.tsx:15-45,47-84</t>
+          <t>src/components/CopyEmailButton.tsx:28-53,63-84</t>
         </is>
       </c>
       <c r="K50" s="13" t="inlineStr">
         <is>
-          <t>src/components/__tests__/CopyEmailButton.test.tsx:29-46; e2e/contact.spec.ts:31-44</t>
+          <t>src/components/__tests__/CopyEmailButton.test.tsx:48-63</t>
         </is>
       </c>
       <c r="L50" s="13" t="inlineStr">
@@ -6463,18 +6481,22 @@
       </c>
       <c r="M50" s="13" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="N50" s="13" t="inlineStr">
         <is>
-          <t>Pass — Controlled clipboard success wrote the exact address, showed Copied/full polite status, then reset after 2.7s. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/interactions/copy-success.png; /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md</t>
-        </is>
-      </c>
-      <c r="O50" s="13" t="n"/>
+          <t>Fail — First failure showed Try copy again/manual guidance, but the second failure produced no live-region mutation or re-announcement. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/interactions/copy-failure-repeat.png; /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md</t>
+        </is>
+      </c>
+      <c r="O50" s="13" t="inlineStr">
+        <is>
+          <t>A11Y-CLIP-001</t>
+        </is>
+      </c>
       <c r="P50" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="Q50" s="13" t="inlineStr">
@@ -6484,7 +6506,7 @@
       </c>
       <c r="R50" s="13" t="inlineStr">
         <is>
-          <t>Pass — Controlled clipboard success wrote the exact address, announced success, changed the button to Copied, and reset after 2.6 seconds; exact-768 success also passed. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-copy-success.png; /tmp/portfolio-feature-audit/postfix/contact-system/lane-c-trace.zip</t>
+          <t>Pass — Controlled consecutive failures produced truthful recovery guidance and distinct polite live-region text for attempts 1 and 2 at 390 and 1440. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-copy-failure-repeat.png; /tmp/portfolio-feature-audit/postfix/contact-system/contact-1440-validation-copy-repeat.png</t>
         </is>
       </c>
       <c r="S50" s="13" t="inlineStr"/>
@@ -6503,7 +6525,7 @@
     <row r="51">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>PF-CONTACT-005</t>
+          <t>PF-CONTACT-006</t>
         </is>
       </c>
       <c r="B51" s="13" t="inlineStr">
@@ -6513,47 +6535,47 @@
       </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
-          <t>/contact clipboard failure</t>
+          <t>/contact draft fields/options</t>
         </is>
       </c>
       <c r="D51" s="13" t="inlineStr">
         <is>
-          <t>Visitor</t>
+          <t>Prospect</t>
         </is>
       </c>
       <c r="E51" s="13" t="inlineStr">
         <is>
-          <t>As a visitor, I want recoverable feedback if copy fails.</t>
+          <t>As a prospect, I want to structure an inquiry.</t>
         </is>
       </c>
       <c r="F51" s="13" t="inlineStr">
         <is>
-          <t>Clipboard API missing/rejects.</t>
+          <t>Contact composer rendered.</t>
         </is>
       </c>
       <c r="G51" s="13" t="inlineStr">
         <is>
-          <t>Activate copy.</t>
+          <t>Enter name/email/message and choose project type/budget.</t>
         </is>
       </c>
       <c r="H51" s="13" t="inlineStr">
         <is>
-          <t>Button becomes “Try copy again” and status advises manual selection; no alert dialog.</t>
+          <t>Offer project types: New website, Portfolio refresh, Cleanup or rescue, Internal tool, Something else; budgets: Under $5k, $5k-$10k, $10k-$25k, $25k+, Not sure yet.</t>
         </is>
       </c>
       <c r="I51" s="13" t="inlineStr">
         <is>
-          <t>Polite live status; amber icon plus text.</t>
+          <t>Labels, required markers, hints, autocomplete/inputMode; two columns at md, message spans both.</t>
         </is>
       </c>
       <c r="J51" s="13" t="inlineStr">
         <is>
-          <t>src/components/CopyEmailButton.tsx:28-53,63-84</t>
+          <t>src/components/ContactComposer.tsx:10-49,178-273</t>
         </is>
       </c>
       <c r="K51" s="13" t="inlineStr">
         <is>
-          <t>src/components/__tests__/CopyEmailButton.test.tsx:48-63</t>
+          <t>src/components/__tests__/ContactComposer.test.tsx:16-38; e2e/contact.spec.ts:46-71</t>
         </is>
       </c>
       <c r="L51" s="13" t="inlineStr">
@@ -6568,12 +6590,12 @@
       </c>
       <c r="N51" s="13" t="inlineStr">
         <is>
-          <t>Fail — First failure showed Try copy again/manual guidance, but the second failure produced no live-region mutation or re-announcement. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/interactions/copy-failure-repeat.png; /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md</t>
+          <t>Fail — Fields/options and md form columns passed, but the desktop sticky explainer moved beneath the fixed dock with 74.41px overlap at 1440px. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/1440/sticky-overlap.png; /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md</t>
         </is>
       </c>
       <c r="O51" s="13" t="inlineStr">
         <is>
-          <t>A11Y-CLIP-001</t>
+          <t>UX-CONTACT-002; RESP-CONTACT-001</t>
         </is>
       </c>
       <c r="P51" s="13" t="inlineStr">
@@ -6588,7 +6610,7 @@
       </c>
       <c r="R51" s="13" t="inlineStr">
         <is>
-          <t>Pass — Controlled consecutive failures produced truthful recovery guidance and distinct polite live-region text for attempts 1 and 2 at 390 and 1440. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-copy-failure-repeat.png; /tmp/portfolio-feature-audit/postfix/contact-system/contact-1440-validation-copy-repeat.png</t>
+          <t>Pass — Correct fields/options and responsive columns rendered. Exact 768 used two columns; pinned 1440x700 explainer had 52px dock clearance and zero overlap. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-768.png; /tmp/portfolio-feature-audit/postfix/contact-system/contact-1440x700-sticky-pinned.png</t>
         </is>
       </c>
       <c r="S51" s="13" t="inlineStr"/>
@@ -6607,7 +6629,7 @@
     <row r="52">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>PF-CONTACT-006</t>
+          <t>PF-CONTACT-007</t>
         </is>
       </c>
       <c r="B52" s="13" t="inlineStr">
@@ -6617,47 +6639,47 @@
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>/contact draft fields/options</t>
+          <t>/contact field validation</t>
         </is>
       </c>
       <c r="D52" s="13" t="inlineStr">
         <is>
-          <t>Prospect</t>
+          <t>Prospect/assistive tech</t>
         </is>
       </c>
       <c r="E52" s="13" t="inlineStr">
         <is>
-          <t>As a prospect, I want to structure an inquiry.</t>
+          <t>As a prospect, I want immediate, specific validation.</t>
         </is>
       </c>
       <c r="F52" s="13" t="inlineStr">
         <is>
-          <t>Contact composer rendered.</t>
+          <t>Field blurred or submit attempted.</t>
         </is>
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>Enter name/email/message and choose project type/budget.</t>
+          <t>Leave blank, enter bad email/unknown option, or message under 10 chars.</t>
         </is>
       </c>
       <c r="H52" s="13" t="inlineStr">
         <is>
-          <t>Offer project types: New website, Portfolio refresh, Cleanup or rescue, Internal tool, Something else; budgets: Under $5k, $5k-$10k, $10k-$25k, $25k+, Not sure yet.</t>
+          <t>Show field-specific message; mark invalid; associate hint/error IDs; revalidate touched fields on change.</t>
         </is>
       </c>
       <c r="I52" s="13" t="inlineStr">
         <is>
-          <t>Labels, required markers, hints, autocomplete/inputMode; two columns at md, message spans both.</t>
+          <t>aria-invalid, aria-describedby, visible rose border/text; no native validation bubble (noValidate).</t>
         </is>
       </c>
       <c r="J52" s="13" t="inlineStr">
         <is>
-          <t>src/components/ContactComposer.tsx:10-49,178-273</t>
+          <t>src/components/ContactComposer.tsx:84-104,178-184,312-440</t>
         </is>
       </c>
       <c r="K52" s="13" t="inlineStr">
         <is>
-          <t>src/components/__tests__/ContactComposer.test.tsx:16-38; e2e/contact.spec.ts:46-71</t>
+          <t>src/components/__tests__/ContactComposer.test.tsx:16-38,90-118; e2e/contact.spec.ts:31-37</t>
         </is>
       </c>
       <c r="L52" s="13" t="inlineStr">
@@ -6672,12 +6694,12 @@
       </c>
       <c r="N52" s="13" t="inlineStr">
         <is>
-          <t>Fail — Fields/options and md form columns passed, but the desktop sticky explainer moved beneath the fixed dock with 74.41px overlap at 1440px. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/1440/sticky-overlap.png; /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md</t>
+          <t>Fail — Blank, bad email, unknown options, under-10 message, and touched-field revalidation passed; all text fields remained unbounded and a 5,000-character message was accepted into a 5,367-character URL. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/validation/empty-submit.png; /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md</t>
         </is>
       </c>
       <c r="O52" s="13" t="inlineStr">
         <is>
-          <t>UX-CONTACT-002; RESP-CONTACT-001</t>
+          <t>UX-CONTACT-002</t>
         </is>
       </c>
       <c r="P52" s="13" t="inlineStr">
@@ -6692,7 +6714,7 @@
       </c>
       <c r="R52" s="13" t="inlineStr">
         <is>
-          <t>Pass — Correct fields/options and responsive columns rendered. Exact 768 used two columns; pinned 1440x700 explainer had 52px dock clearance and zero overlap. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-768.png; /tmp/portfolio-feature-audit/postfix/contact-system/contact-1440x700-sticky-pinned.png</t>
+          <t>Pass — Specific blank/email/message validation, aria associations, and touched revalidation passed. Name/email/message limits are 80/254/1000; overfill truncated to 1000 with a live counter. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-validation-empty.png; /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-url-limit.png</t>
         </is>
       </c>
       <c r="S52" s="13" t="inlineStr"/>
@@ -6711,7 +6733,7 @@
     <row r="53">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>PF-CONTACT-007</t>
+          <t>PF-CONTACT-008</t>
         </is>
       </c>
       <c r="B53" s="13" t="inlineStr">
@@ -6721,47 +6743,47 @@
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>/contact field validation</t>
+          <t>/contact invalid-submit focus</t>
         </is>
       </c>
       <c r="D53" s="13" t="inlineStr">
         <is>
-          <t>Prospect/assistive tech</t>
+          <t>Prospect/keyboard user</t>
         </is>
       </c>
       <c r="E53" s="13" t="inlineStr">
         <is>
-          <t>As a prospect, I want immediate, specific validation.</t>
+          <t>As a prospect, I want errors summarized and focus moved to the first problem.</t>
         </is>
       </c>
       <c r="F53" s="13" t="inlineStr">
         <is>
-          <t>Field blurred or submit attempted.</t>
+          <t>Form contains any invalid field.</t>
         </is>
       </c>
       <c r="G53" s="13" t="inlineStr">
         <is>
-          <t>Leave blank, enter bad email/unknown option, or message under 10 chars.</t>
+          <t>Submit.</t>
         </is>
       </c>
       <c r="H53" s="13" t="inlineStr">
         <is>
-          <t>Show field-specific message; mark invalid; associate hint/error IDs; revalidate touched fields on change.</t>
+          <t>Prevent draft, mark all touched, set error status, focus first invalid field in field order.</t>
         </is>
       </c>
       <c r="I53" s="13" t="inlineStr">
         <is>
-          <t>aria-invalid, aria-describedby, visible rose border/text; no native validation bubble (noValidate).</t>
+          <t>Assertive alert status on error; deterministic focus recovery.</t>
         </is>
       </c>
       <c r="J53" s="13" t="inlineStr">
         <is>
-          <t>src/components/ContactComposer.tsx:84-104,178-184,312-440</t>
+          <t>src/components/ContactComposer.tsx:106-143,299-306,446-462</t>
         </is>
       </c>
       <c r="K53" s="13" t="inlineStr">
         <is>
-          <t>src/components/__tests__/ContactComposer.test.tsx:16-38,90-118; e2e/contact.spec.ts:31-37</t>
+          <t>src/components/__tests__/ContactComposer.test.tsx:16-38,90-118; E2E checks invalid state but not focus e2e/contact.spec.ts:31-37</t>
         </is>
       </c>
       <c r="L53" s="13" t="inlineStr">
@@ -6771,22 +6793,18 @@
       </c>
       <c r="M53" s="13" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="N53" s="13" t="inlineStr">
         <is>
-          <t>Fail — Blank, bad email, unknown options, under-10 message, and touched-field revalidation passed; all text fields remained unbounded and a 5,000-character message was accepted into a 5,367-character URL. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/validation/empty-submit.png; /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md</t>
-        </is>
-      </c>
-      <c r="O53" s="13" t="inlineStr">
-        <is>
-          <t>UX-CONTACT-002</t>
-        </is>
-      </c>
+          <t>Pass — All fields became invalid, atomic assertive summary appeared, no mailto was created, and focus moved to Your name. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/validation/empty-submit.png; /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md</t>
+        </is>
+      </c>
+      <c r="O53" s="13" t="n"/>
       <c r="P53" s="13" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="Q53" s="13" t="inlineStr">
@@ -6796,7 +6814,7 @@
       </c>
       <c r="R53" s="13" t="inlineStr">
         <is>
-          <t>Pass — Specific blank/email/message validation, aria associations, and touched revalidation passed. Name/email/message limits are 80/254/1000; overfill truncated to 1000 with a live counter. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-validation-empty.png; /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-url-limit.png</t>
+          <t>Pass — Empty submit marked five fields invalid, emitted an assertive alert, created no mailto, and focused Your name at 390, 768, and 1440. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-validation-empty.png; /tmp/portfolio-feature-audit/postfix/contact-system/contact-1440-validation-copy-repeat.png</t>
         </is>
       </c>
       <c r="S53" s="13" t="inlineStr"/>
@@ -6815,7 +6833,7 @@
     <row r="54">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>PF-CONTACT-008</t>
+          <t>PF-CONTACT-009</t>
         </is>
       </c>
       <c r="B54" s="13" t="inlineStr">
@@ -6825,47 +6843,47 @@
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>/contact invalid-submit focus</t>
+          <t>/contact encoded mailto draft</t>
         </is>
       </c>
       <c r="D54" s="13" t="inlineStr">
         <is>
-          <t>Prospect/keyboard user</t>
+          <t>Prospect</t>
         </is>
       </c>
       <c r="E54" s="13" t="inlineStr">
         <is>
-          <t>As a prospect, I want errors summarized and focus moved to the first problem.</t>
+          <t>As a prospect, I want a reviewable draft, not automatic sending.</t>
         </is>
       </c>
       <c r="F54" s="13" t="inlineStr">
         <is>
-          <t>Form contains any invalid field.</t>
+          <t>All fields valid and mail client available.</t>
         </is>
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>Submit.</t>
+          <t>Activate “Prepare email draft.”</t>
         </is>
       </c>
       <c r="H54" s="13" t="inlineStr">
         <is>
-          <t>Prevent draft, mark all touched, set error status, focus first invalid field in field order.</t>
+          <t>Trim inputs; build encoded subject/body with labels and provenance; programmatically click protected mailto:; nothing sends automatically.</t>
         </is>
       </c>
       <c r="I54" s="13" t="inlineStr">
         <is>
-          <t>Assertive alert status on error; deterministic focus recovery.</t>
+          <t>Submit disabled/aria-busy while preparing; visible spinner and explicit status.</t>
         </is>
       </c>
       <c r="J54" s="13" t="inlineStr">
         <is>
-          <t>src/components/ContactComposer.tsx:106-143,299-306,446-462</t>
+          <t>src/components/ContactComposer.tsx:51-68,106-169,275-308</t>
         </is>
       </c>
       <c r="K54" s="13" t="inlineStr">
         <is>
-          <t>src/components/__tests__/ContactComposer.test.tsx:16-38,90-118; E2E checks invalid state but not focus e2e/contact.spec.ts:31-37</t>
+          <t>src/components/__tests__/ContactComposer.test.tsx:40-88; e2e/contact.spec.ts:46-71</t>
         </is>
       </c>
       <c r="L54" s="13" t="inlineStr">
@@ -6875,18 +6893,22 @@
       </c>
       <c r="M54" s="13" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="N54" s="13" t="inlineStr">
         <is>
-          <t>Pass — All fields became invalid, atomic assertive summary appeared, no mailto was created, and focus moved to Your name. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/validation/empty-submit.png; /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md</t>
-        </is>
-      </c>
-      <c r="O54" s="13" t="n"/>
+          <t>Fail — Encoded protected mailto was correct and safely intercepted, but MutationObserver saw idle jump directly to success; aria-busy, spinner, and Preparing draft never rendered. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/interactions/valid-mailto-intercept.png; /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md</t>
+        </is>
+      </c>
+      <c r="O54" s="13" t="inlineStr">
+        <is>
+          <t>UX-CONTACT-001; UX-CONTACT-002; BL-SYS-001</t>
+        </is>
+      </c>
       <c r="P54" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="Q54" s="13" t="inlineStr">
@@ -6896,7 +6918,7 @@
       </c>
       <c r="R54" s="13" t="inlineStr">
         <is>
-          <t>Pass — Empty submit marked five fields invalid, emitted an assertive alert, created no mailto, and focused Your name at 390, 768, and 1440. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-validation-empty.png; /tmp/portfolio-feature-audit/postfix/contact-system/contact-1440-validation-copy-repeat.png</t>
+          <t>Pass — Valid input generated one correctly encoded intercepted mailto. Busy, disabled, spinner, and Preparing state were observable for about 302ms. Oversize encoded URL was rejected before handoff and focused Message. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-preparing.png; /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-mailto-neutral.png; /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-url-limit.png</t>
         </is>
       </c>
       <c r="S54" s="13" t="inlineStr"/>
@@ -6915,7 +6937,7 @@
     <row r="55">
       <c r="A55" s="13" t="inlineStr">
         <is>
-          <t>PF-CONTACT-009</t>
+          <t>PF-CONTACT-010</t>
         </is>
       </c>
       <c r="B55" s="13" t="inlineStr">
@@ -6925,47 +6947,47 @@
       </c>
       <c r="C55" s="13" t="inlineStr">
         <is>
-          <t>/contact encoded mailto draft</t>
+          <t>/contact inquiry analytics</t>
         </is>
       </c>
       <c r="D55" s="13" t="inlineStr">
         <is>
-          <t>Prospect</t>
+          <t>Site operator</t>
         </is>
       </c>
       <c r="E55" s="13" t="inlineStr">
         <is>
-          <t>As a prospect, I want a reviewable draft, not automatic sending.</t>
+          <t>As an operator, I want privacy-minimal draft intent telemetry.</t>
         </is>
       </c>
       <c r="F55" s="13" t="inlineStr">
         <is>
-          <t>All fields valid and mail client available.</t>
+          <t>Valid draft action in browser production runtime.</t>
         </is>
       </c>
       <c r="G55" s="13" t="inlineStr">
         <is>
-          <t>Activate “Prepare email draft.”</t>
+          <t>Prepare draft.</t>
         </is>
       </c>
       <c r="H55" s="13" t="inlineStr">
         <is>
-          <t>Trim inputs; build encoded subject/body with labels and provenance; programmatically click protected mailto:; nothing sends automatically.</t>
+          <t>Track contact_mailto_draft with only project type and budget; drop null/undefined properties; failures do not block UX.</t>
         </is>
       </c>
       <c r="I55" s="13" t="inlineStr">
         <is>
-          <t>Submit disabled/aria-busy while preparing; visible spinner and explicit status.</t>
+          <t>No name/email/message sent; fail-closed in test/server/unavailable runtime.</t>
         </is>
       </c>
       <c r="J55" s="13" t="inlineStr">
         <is>
-          <t>src/components/ContactComposer.tsx:51-68,106-169,275-308</t>
+          <t>src/components/ContactComposer.tsx:145-149; src/utils/analytics.ts:10-36</t>
         </is>
       </c>
       <c r="K55" s="13" t="inlineStr">
         <is>
-          <t>src/components/__tests__/ContactComposer.test.tsx:40-88; e2e/contact.spec.ts:46-71</t>
+          <t>src/components/__tests__/ContactComposer.test.tsx:40-88,120-148</t>
         </is>
       </c>
       <c r="L55" s="13" t="inlineStr">
@@ -6975,22 +6997,18 @@
       </c>
       <c r="M55" s="13" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="N55" s="13" t="inlineStr">
         <is>
-          <t>Fail — Encoded protected mailto was correct and safely intercepted, but MutationObserver saw idle jump directly to success; aria-busy, spinner, and Preparing draft never rendered. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/interactions/valid-mailto-intercept.png; /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md</t>
-        </is>
-      </c>
-      <c r="O55" s="13" t="inlineStr">
-        <is>
-          <t>UX-CONTACT-001; UX-CONTACT-002; BL-SYS-001</t>
-        </is>
-      </c>
+          <t>Pass — Runtime window.va capture contained only project_type and budget_range; source/tests drop null/undefined and catch runtime failures. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md; /tmp/portfolio-feature-audit/baseline/contact-system/validation-evidence.md</t>
+        </is>
+      </c>
+      <c r="O55" s="13" t="n"/>
       <c r="P55" s="13" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="Q55" s="13" t="inlineStr">
@@ -7000,7 +7018,7 @@
       </c>
       <c r="R55" s="13" t="inlineStr">
         <is>
-          <t>Pass — Valid input generated one correctly encoded intercepted mailto. Busy, disabled, spinner, and Preparing state were observable for about 302ms. Oversize encoded URL was rejected before handoff and focused Message. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-preparing.png; /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-mailto-neutral.png; /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-url-limit.png</t>
+          <t>Pass — Captured contact_mailto_draft event contained only project_type and budget_range; no personal fields were included. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/lane-c-trace.zip; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
         </is>
       </c>
       <c r="S55" s="13" t="inlineStr"/>
@@ -7019,7 +7037,7 @@
     <row r="56">
       <c r="A56" s="13" t="inlineStr">
         <is>
-          <t>PF-CONTACT-010</t>
+          <t>PF-CONTACT-011</t>
         </is>
       </c>
       <c r="B56" s="13" t="inlineStr">
@@ -7029,47 +7047,47 @@
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>/contact inquiry analytics</t>
+          <t>/contact form status announcements</t>
         </is>
       </c>
       <c r="D56" s="13" t="inlineStr">
         <is>
-          <t>Site operator</t>
+          <t>Prospect/assistive tech</t>
         </is>
       </c>
       <c r="E56" s="13" t="inlineStr">
         <is>
-          <t>As an operator, I want privacy-minimal draft intent telemetry.</t>
+          <t>As a user, I want clear idle/preparing/success/error state.</t>
         </is>
       </c>
       <c r="F56" s="13" t="inlineStr">
         <is>
-          <t>Valid draft action in browser production runtime.</t>
+          <t>Composer rendered/submitted.</t>
         </is>
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>Prepare draft.</t>
+          <t>Interact with form.</t>
         </is>
       </c>
       <c r="H56" s="13" t="inlineStr">
         <is>
-          <t>Track contact_mailto_draft with only project type and budget; drop null/undefined properties; failures do not block UX.</t>
+          <t>Announce “nothing sent,” preparing, success, or validation error; success says mail app should open.</t>
         </is>
       </c>
       <c r="I56" s="13" t="inlineStr">
         <is>
-          <t>No name/email/message sent; fail-closed in test/server/unavailable runtime.</t>
+          <t>role=status polite normally; role=alert assertive on error; atomic.</t>
         </is>
       </c>
       <c r="J56" s="13" t="inlineStr">
         <is>
-          <t>src/components/ContactComposer.tsx:145-149; src/utils/analytics.ts:10-36</t>
+          <t>src/components/ContactComposer.tsx:162-176,299-306</t>
         </is>
       </c>
       <c r="K56" s="13" t="inlineStr">
         <is>
-          <t>src/components/__tests__/ContactComposer.test.tsx:40-88,120-148</t>
+          <t>src/components/__tests__/ContactComposer.test.tsx:90-118; e2e/contact.spec.ts:34,55-57</t>
         </is>
       </c>
       <c r="L56" s="13" t="inlineStr">
@@ -7079,18 +7097,22 @@
       </c>
       <c r="M56" s="13" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="N56" s="13" t="inlineStr">
         <is>
-          <t>Pass — Runtime window.va capture contained only project_type and budget_range; source/tests drop null/undefined and catch runtime failures. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md; /tmp/portfolio-feature-audit/baseline/contact-system/validation-evidence.md</t>
-        </is>
-      </c>
-      <c r="O56" s="13" t="n"/>
+          <t>Fail — Idle and validation alert semantics passed, but preparing never rendered and a no-op intercepted protocol click immediately claimed the mail app should open. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md; /tmp/portfolio-feature-audit/baseline/contact-system/interactions/valid-mailto-intercept.png</t>
+        </is>
+      </c>
+      <c r="O56" s="13" t="inlineStr">
+        <is>
+          <t>UX-CONTACT-001; BL-SYS-001</t>
+        </is>
+      </c>
       <c r="P56" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="Q56" s="13" t="inlineStr">
@@ -7100,7 +7122,7 @@
       </c>
       <c r="R56" s="13" t="inlineStr">
         <is>
-          <t>Pass — Captured contact_mailto_draft event contained only project_type and budget_range; no personal fields were included. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/lane-c-trace.zip; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
+          <t>Pass — Idle, assertive validation, polite preparing, and neutral completion semantics passed; completion explicitly states Email draft requested and Nothing was sent with fallbacks. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-preparing.png; /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-mailto-neutral.png</t>
         </is>
       </c>
       <c r="S56" s="13" t="inlineStr"/>
@@ -7119,7 +7141,7 @@
     <row r="57">
       <c r="A57" s="13" t="inlineStr">
         <is>
-          <t>PF-CONTACT-011</t>
+          <t>PF-CONTACT-012</t>
         </is>
       </c>
       <c r="B57" s="13" t="inlineStr">
@@ -7129,47 +7151,47 @@
       </c>
       <c r="C57" s="13" t="inlineStr">
         <is>
-          <t>/contact form status announcements</t>
+          <t>/contact secondary channels</t>
         </is>
       </c>
       <c r="D57" s="13" t="inlineStr">
         <is>
-          <t>Prospect/assistive tech</t>
+          <t>Visitor</t>
         </is>
       </c>
       <c r="E57" s="13" t="inlineStr">
         <is>
-          <t>As a user, I want clear idle/preparing/success/error state.</t>
+          <t>As a visitor, I want professional alternatives.</t>
         </is>
       </c>
       <c r="F57" s="13" t="inlineStr">
         <is>
-          <t>Composer rendered/submitted.</t>
+          <t>Secondary contact list rendered.</t>
         </is>
       </c>
       <c r="G57" s="13" t="inlineStr">
         <is>
-          <t>Interact with form.</t>
+          <t>Activate GitHub, LinkedIn, or Defendre Solutions card.</t>
         </is>
       </c>
       <c r="H57" s="13" t="inlineStr">
         <is>
-          <t>Announce “nothing sent,” preparing, success, or validation error; success says mail app should open.</t>
+          <t>Open configured external destination in protected new tab.</t>
         </is>
       </c>
       <c r="I57" s="13" t="inlineStr">
         <is>
-          <t>role=status polite normally; role=alert assertive on error; atomic.</t>
+          <t>Large focusable cards; icon decorative; visible name/description/value.</t>
         </is>
       </c>
       <c r="J57" s="13" t="inlineStr">
         <is>
-          <t>src/components/ContactComposer.tsx:162-176,299-306</t>
+          <t>src/data/socials.ts:40-64; src/app/(site)/contact/page.tsx:128-181</t>
         </is>
       </c>
       <c r="K57" s="13" t="inlineStr">
         <is>
-          <t>src/components/__tests__/ContactComposer.test.tsx:90-118; e2e/contact.spec.ts:34,55-57</t>
+          <t>src/app/(site)/contact/page.test.tsx:27-51; src/data/__tests__/socials.test.ts:41-76</t>
         </is>
       </c>
       <c r="L57" s="13" t="inlineStr">
@@ -7184,12 +7206,12 @@
       </c>
       <c r="N57" s="13" t="inlineStr">
         <is>
-          <t>Fail — Idle and validation alert semantics passed, but preparing never rendered and a no-op intercepted protocol click immediately claimed the mail app should open. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md; /tmp/portfolio-feature-audit/baseline/contact-system/interactions/valid-mailto-intercept.png</t>
+          <t>Fail — Destinations, target, rel, and large geometry passed, but accessible names omit the new-tab context change. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md; /tmp/portfolio-feature-audit/baseline/contact-system/snapshot-contact-390.txt</t>
         </is>
       </c>
       <c r="O57" s="13" t="inlineStr">
         <is>
-          <t>UX-CONTACT-001; BL-SYS-001</t>
+          <t>A11Y-EXT-001; DESIGN-AI-001</t>
         </is>
       </c>
       <c r="P57" s="13" t="inlineStr">
@@ -7204,7 +7226,7 @@
       </c>
       <c r="R57" s="13" t="inlineStr">
         <is>
-          <t>Pass — Idle, assertive validation, polite preparing, and neutral completion semantics passed; completion explicitly states Email draft requested and Nothing was sent with fallbacks. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-preparing.png; /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-mailto-neutral.png</t>
+          <t>Pass — GitHub, LinkedIn, and studio cards retained correct protected new-tab destinations and now disclose opens in a new tab in accessible names. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/lane-c-trace.zip; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
         </is>
       </c>
       <c r="S57" s="13" t="inlineStr"/>
@@ -7223,7 +7245,7 @@
     <row r="58">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>PF-CONTACT-012</t>
+          <t>PF-CONTACT-013</t>
         </is>
       </c>
       <c r="B58" s="13" t="inlineStr">
@@ -7233,47 +7255,47 @@
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>/contact secondary channels</t>
+          <t>/contact LinkedIn responsive label</t>
         </is>
       </c>
       <c r="D58" s="13" t="inlineStr">
         <is>
-          <t>Visitor</t>
+          <t>Mobile visitor</t>
         </is>
       </c>
       <c r="E58" s="13" t="inlineStr">
         <is>
-          <t>As a visitor, I want professional alternatives.</t>
+          <t>As a mobile visitor, I want a non-overflowing LinkedIn label.</t>
         </is>
       </c>
       <c r="F58" s="13" t="inlineStr">
         <is>
-          <t>Secondary contact list rendered.</t>
+          <t>Secondary LinkedIn card visible.</t>
         </is>
       </c>
       <c r="G58" s="13" t="inlineStr">
         <is>
-          <t>Activate GitHub, LinkedIn, or Defendre Solutions card.</t>
+          <t>View below/above sm.</t>
         </is>
       </c>
       <c r="H58" s="13" t="inlineStr">
         <is>
-          <t>Open configured external destination in protected new tab.</t>
+          <t>Show “LinkedIn profile” on mobile and full path at sm+.</t>
         </is>
       </c>
       <c r="I58" s="13" t="inlineStr">
         <is>
-          <t>Large focusable cards; icon decorative; visible name/description/value.</t>
+          <t>Prevents long label overflow without changing destination/name.</t>
         </is>
       </c>
       <c r="J58" s="13" t="inlineStr">
         <is>
-          <t>src/data/socials.ts:40-64; src/app/(site)/contact/page.tsx:128-181</t>
+          <t>src/data/socials.ts:49-55; src/app/(site)/contact/page.tsx:168-177</t>
         </is>
       </c>
       <c r="K58" s="13" t="inlineStr">
         <is>
-          <t>src/app/(site)/contact/page.test.tsx:27-51; src/data/__tests__/socials.test.ts:41-76</t>
+          <t>/contact mobile overflow e2e/contact.spec.ts:43; no direct label assertion</t>
         </is>
       </c>
       <c r="L58" s="13" t="inlineStr">
@@ -7283,22 +7305,18 @@
       </c>
       <c r="M58" s="13" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="N58" s="13" t="inlineStr">
         <is>
-          <t>Fail — Destinations, target, rel, and large geometry passed, but accessible names omit the new-tab context change. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md; /tmp/portfolio-feature-audit/baseline/contact-system/snapshot-contact-390.txt</t>
-        </is>
-      </c>
-      <c r="O58" s="13" t="inlineStr">
-        <is>
-          <t>A11Y-EXT-001; DESIGN-AI-001</t>
-        </is>
-      </c>
+          <t>Pass — LinkedIn profile displayed at 390; full path displayed at 768+; no horizontal overflow. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/390/contact-full.png; /tmp/portfolio-feature-audit/baseline/contact-system/768/contact-full.png</t>
+        </is>
+      </c>
+      <c r="O58" s="13" t="n"/>
       <c r="P58" s="13" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="Q58" s="13" t="inlineStr">
@@ -7308,7 +7326,7 @@
       </c>
       <c r="R58" s="13" t="inlineStr">
         <is>
-          <t>Pass — GitHub, LinkedIn, and studio cards retained correct protected new-tab destinations and now disclose opens in a new tab in accessible names. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/lane-c-trace.zip; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
+          <t>Pass — LinkedIn profile was the only visible value at 390; full profile path was the only visible value at exact 768; no overflow occurred. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-initial.png; /tmp/portfolio-feature-audit/postfix/contact-system/contact-768.png</t>
         </is>
       </c>
       <c r="S58" s="13" t="inlineStr"/>
@@ -7327,7 +7345,7 @@
     <row r="59">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>PF-CONTACT-013</t>
+          <t>PF-CONTACT-014</t>
         </is>
       </c>
       <c r="B59" s="13" t="inlineStr">
@@ -7337,47 +7355,47 @@
       </c>
       <c r="C59" s="13" t="inlineStr">
         <is>
-          <t>/contact LinkedIn responsive label</t>
+          <t>/contact low-priority support</t>
         </is>
       </c>
       <c r="D59" s="13" t="inlineStr">
         <is>
-          <t>Mobile visitor</t>
+          <t>Supporter</t>
         </is>
       </c>
       <c r="E59" s="13" t="inlineStr">
         <is>
-          <t>As a mobile visitor, I want a non-overflowing LinkedIn label.</t>
+          <t>As a supporter, I want an optional support link without displacing inquiry CTAs.</t>
         </is>
       </c>
       <c r="F59" s="13" t="inlineStr">
         <is>
-          <t>Secondary LinkedIn card visible.</t>
+          <t>Footer-priority link exists.</t>
         </is>
       </c>
       <c r="G59" s="13" t="inlineStr">
         <is>
-          <t>View below/above sm.</t>
+          <t>Activate “Support.”</t>
         </is>
       </c>
       <c r="H59" s="13" t="inlineStr">
         <is>
-          <t>Show “LinkedIn profile” on mobile and full path at sm+.</t>
+          <t>Open Buy Me a Coffee in protected new tab from footer/studio panel.</t>
         </is>
       </c>
       <c r="I59" s="13" t="inlineStr">
         <is>
-          <t>Prevents long label overflow without changing destination/name.</t>
+          <t>44px focusable pill; labelled “Support Defendre Solutions”; deliberately not primary/social nav.</t>
         </is>
       </c>
       <c r="J59" s="13" t="inlineStr">
         <is>
-          <t>src/data/socials.ts:49-55; src/app/(site)/contact/page.tsx:168-177</t>
+          <t>src/data/socials.ts:22-29,65; src/app/(site)/contact/page.tsx:184-213</t>
         </is>
       </c>
       <c r="K59" s="13" t="inlineStr">
         <is>
-          <t>/contact mobile overflow e2e/contact.spec.ts:43; no direct label assertion</t>
+          <t>src/app/(site)/contact/page.test.tsx:52-59; src/data/__tests__/socials.test.ts:34-39,73-76</t>
         </is>
       </c>
       <c r="L59" s="13" t="inlineStr">
@@ -7387,18 +7405,22 @@
       </c>
       <c r="M59" s="13" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="N59" s="13" t="inlineStr">
         <is>
-          <t>Pass — LinkedIn profile displayed at 390; full path displayed at 768+; no horizontal overflow. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/390/contact-full.png; /tmp/portfolio-feature-audit/baseline/contact-system/768/contact-full.png</t>
-        </is>
-      </c>
-      <c r="O59" s="13" t="n"/>
+          <t>Fail — Placement, label, 44px target, and destination passed, but its accessible name omits the new-tab context change. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md; /tmp/portfolio-feature-audit/baseline/contact-system/1440/contact-full.png</t>
+        </is>
+      </c>
+      <c r="O59" s="13" t="inlineStr">
+        <is>
+          <t>A11Y-EXT-001; DESIGN-AI-001</t>
+        </is>
+      </c>
       <c r="P59" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="Q59" s="13" t="inlineStr">
@@ -7408,7 +7430,7 @@
       </c>
       <c r="R59" s="13" t="inlineStr">
         <is>
-          <t>Pass — LinkedIn profile was the only visible value at 390; full profile path was the only visible value at exact 768; no overflow occurred. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-390-initial.png; /tmp/portfolio-feature-audit/postfix/contact-system/contact-768.png</t>
+          <t>Pass — Support remained footer-priority with a 44px target, correct URL, protected new tab, and disclosed context-change accessible name. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-1440-validation-copy-repeat.png; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
         </is>
       </c>
       <c r="S59" s="13" t="inlineStr"/>
@@ -7427,7 +7449,7 @@
     <row r="60">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>PF-CONTACT-014</t>
+          <t>PF-404-001</t>
         </is>
       </c>
       <c r="B60" s="13" t="inlineStr">
@@ -7437,47 +7459,47 @@
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>/contact low-priority support</t>
+          <t>Custom not found</t>
         </is>
       </c>
       <c r="D60" s="13" t="inlineStr">
         <is>
-          <t>Supporter</t>
+          <t>Lost visitor</t>
         </is>
       </c>
       <c r="E60" s="13" t="inlineStr">
         <is>
-          <t>As a supporter, I want an optional support link without displacing inquiry CTAs.</t>
+          <t>As a visitor on a bad route, I want a branded explanation.</t>
         </is>
       </c>
       <c r="F60" s="13" t="inlineStr">
         <is>
-          <t>Footer-priority link exists.</t>
+          <t>Framework resolves unmatched route.</t>
         </is>
       </c>
       <c r="G60" s="13" t="inlineStr">
         <is>
-          <t>Activate “Support.”</t>
+          <t>Load unknown URL.</t>
         </is>
       </c>
       <c r="H60" s="13" t="inlineStr">
         <is>
-          <t>Open Buy Me a Coffee in protected new tab from footer/studio panel.</t>
+          <t>Render Page not found, signal-lost narrative, 404 decoration, normal ambient/navigation shell, and route-specific metadata.</t>
         </is>
       </c>
       <c r="I60" s="13" t="inlineStr">
         <is>
-          <t>44px focusable pill; labelled “Support Defendre Solutions”; deliberately not primary/social nav.</t>
+          <t>Semantic h1; decorative 404 hidden; responsive panel; skip link.</t>
         </is>
       </c>
       <c r="J60" s="13" t="inlineStr">
         <is>
-          <t>src/data/socials.ts:22-29,65; src/app/(site)/contact/page.tsx:184-213</t>
+          <t>src/app/not-found.tsx:7-11,31-69</t>
         </is>
       </c>
       <c r="K60" s="13" t="inlineStr">
         <is>
-          <t>src/app/(site)/contact/page.test.tsx:52-59; src/data/__tests__/socials.test.ts:34-39,73-76</t>
+          <t>src/app/not-found.test.tsx:27-51</t>
         </is>
       </c>
       <c r="L60" s="13" t="inlineStr">
@@ -7487,22 +7509,18 @@
       </c>
       <c r="M60" s="13" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="N60" s="13" t="inlineStr">
         <is>
-          <t>Fail — Placement, label, 44px target, and destination passed, but its accessible name omits the new-tab context change. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/contact-interactions.md; /tmp/portfolio-feature-audit/baseline/contact-system/1440/contact-full.png</t>
-        </is>
-      </c>
-      <c r="O60" s="13" t="inlineStr">
-        <is>
-          <t>A11Y-EXT-001; DESIGN-AI-001</t>
-        </is>
-      </c>
+          <t>Pass — HTTP response is 404; title is Page Not Found; the Steve Defendre signal-lost message, Page not found h1, explanatory copy, dark shell, and no active primary route render at 390/768/1440 without overflow. Evidence: /tmp/portfolio-feature-audit/baseline/core/not-found-http-headers.txt; /tmp/portfolio-feature-audit/baseline/core/not-found-1440-a11y.txt; /tmp/portfolio-feature-audit/baseline/core/not-found-390-full.png; /tmp/portfolio-feature-audit/baseline/core/not-found-768-full.png; /tmp/portfolio-feature-audit/baseline/core/not-found-1440-full.png</t>
+        </is>
+      </c>
+      <c r="O60" s="13" t="n"/>
       <c r="P60" s="13" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="Q60" s="13" t="inlineStr">
@@ -7512,7 +7530,7 @@
       </c>
       <c r="R60" s="13" t="inlineStr">
         <is>
-          <t>Pass — Support remained footer-priority with a 44px target, correct URL, protected new tab, and disclosed context-change accessible name. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/contact-1440-validation-copy-repeat.png; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
+          <t>Pass — The invalid route rendered Page not found, signal-lost copy, 404 decoration, ambient shell, route title/description, one visible navigation, and no overflow at 390/768/1440. Evidence: /tmp/portfolio-feature-audit/postfix/core/390/not-found-diagnostics.json; /tmp/portfolio-feature-audit/postfix/core/390/not-found-a11y.txt; /tmp/portfolio-feature-audit/postfix/core/390/not-found-full.png; /tmp/portfolio-feature-audit/postfix/core/768/not-found-full.png; /tmp/portfolio-feature-audit/postfix/core/1440/not-found-full.png</t>
         </is>
       </c>
       <c r="S60" s="13" t="inlineStr"/>
@@ -7531,7 +7549,7 @@
     <row r="61">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>PF-404-001</t>
+          <t>PF-404-002</t>
         </is>
       </c>
       <c r="B61" s="13" t="inlineStr">
@@ -7541,7 +7559,7 @@
       </c>
       <c r="C61" s="13" t="inlineStr">
         <is>
-          <t>Custom not found</t>
+          <t>Custom not found recovery</t>
         </is>
       </c>
       <c r="D61" s="13" t="inlineStr">
@@ -7551,37 +7569,37 @@
       </c>
       <c r="E61" s="13" t="inlineStr">
         <is>
-          <t>As a visitor on a bad route, I want a branded explanation.</t>
+          <t>As a lost visitor, I want recovery destinations.</t>
         </is>
       </c>
       <c r="F61" s="13" t="inlineStr">
         <is>
-          <t>Framework resolves unmatched route.</t>
+          <t>404 shown.</t>
         </is>
       </c>
       <c r="G61" s="13" t="inlineStr">
         <is>
-          <t>Load unknown URL.</t>
+          <t>Activate Home, Projects, or Contact.</t>
         </is>
       </c>
       <c r="H61" s="13" t="inlineStr">
         <is>
-          <t>Render Page not found, signal-lost narrative, 404 decoration, normal ambient/navigation shell, and route-specific metadata.</t>
+          <t>Navigate to selected route via recovery nav.</t>
         </is>
       </c>
       <c r="I61" s="13" t="inlineStr">
         <is>
-          <t>Semantic h1; decorative 404 hidden; responsive panel; skip link.</t>
+          <t>nav aria-label="Page recovery"; two-column mobile grid/row at sm; 48px controls.</t>
         </is>
       </c>
       <c r="J61" s="13" t="inlineStr">
         <is>
-          <t>src/app/not-found.tsx:7-11,31-69</t>
+          <t>src/app/not-found.tsx:13-29,70-84</t>
         </is>
       </c>
       <c r="K61" s="13" t="inlineStr">
         <is>
-          <t>src/app/not-found.test.tsx:27-51</t>
+          <t>src/app/not-found.test.tsx:27-46</t>
         </is>
       </c>
       <c r="L61" s="13" t="inlineStr">
@@ -7596,7 +7614,7 @@
       </c>
       <c r="N61" s="13" t="inlineStr">
         <is>
-          <t>Pass — HTTP response is 404; title is Page Not Found; the Steve Defendre signal-lost message, Page not found h1, explanatory copy, dark shell, and no active primary route render at 390/768/1440 without overflow. Evidence: /tmp/portfolio-feature-audit/baseline/core/not-found-http-headers.txt; /tmp/portfolio-feature-audit/baseline/core/not-found-1440-a11y.txt; /tmp/portfolio-feature-audit/baseline/core/not-found-390-full.png; /tmp/portfolio-feature-audit/baseline/core/not-found-768-full.png; /tmp/portfolio-feature-audit/baseline/core/not-found-1440-full.png</t>
+          <t>Pass — Accessibility tree exposes Page recovery navigation; keyboard Home and click Projects/Contact each reached the intended route; mobile controls reflow 2+1 and remain clear of the dock. Evidence: /tmp/portfolio-feature-audit/baseline/core/not-found-1440-a11y.txt; /tmp/portfolio-feature-audit/baseline/core/not-found-recovery-home-keyboard.txt; /tmp/portfolio-feature-audit/baseline/core/not-found-recovery-projects.txt; /tmp/portfolio-feature-audit/baseline/core/not-found-recovery-contact.txt; /tmp/portfolio-feature-audit/baseline/core/not-found-390-full.png</t>
         </is>
       </c>
       <c r="O61" s="13" t="n"/>
@@ -7612,7 +7630,7 @@
       </c>
       <c r="R61" s="13" t="inlineStr">
         <is>
-          <t>Pass — The invalid route rendered Page not found, signal-lost copy, 404 decoration, ambient shell, route title/description, one visible navigation, and no overflow at 390/768/1440. Evidence: /tmp/portfolio-feature-audit/postfix/core/390/not-found-diagnostics.json; /tmp/portfolio-feature-audit/postfix/core/390/not-found-a11y.txt; /tmp/portfolio-feature-audit/postfix/core/390/not-found-full.png; /tmp/portfolio-feature-audit/postfix/core/768/not-found-full.png; /tmp/portfolio-feature-audit/postfix/core/1440/not-found-full.png</t>
+          <t>Pass — The labelled recovery navigation rendered three 47.6px+ targets; each was activated and reached its intended route. Evidence: /tmp/portfolio-feature-audit/postfix/core/390/not-found-diagnostics.json; /tmp/portfolio-feature-audit/postfix/core/390/recovery-home-url.txt; /tmp/portfolio-feature-audit/postfix/core/390/recovery-projects-url.txt; /tmp/portfolio-feature-audit/postfix/core/390/recovery-contact-url.txt</t>
         </is>
       </c>
       <c r="S61" s="13" t="inlineStr"/>
@@ -7631,7 +7649,7 @@
     <row r="62">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>PF-404-002</t>
+          <t>PF-404-003</t>
         </is>
       </c>
       <c r="B62" s="13" t="inlineStr">
@@ -7641,17 +7659,17 @@
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>Custom not found recovery</t>
+          <t>Custom not found attribution/analytics</t>
         </is>
       </c>
       <c r="D62" s="13" t="inlineStr">
         <is>
-          <t>Lost visitor</t>
+          <t>Visitor/operator</t>
         </is>
       </c>
       <c r="E62" s="13" t="inlineStr">
         <is>
-          <t>As a lost visitor, I want recovery destinations.</t>
+          <t>As a visitor/operator, I want attribution and page-view telemetry.</t>
         </is>
       </c>
       <c r="F62" s="13" t="inlineStr">
@@ -7661,27 +7679,27 @@
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>Activate Home, Projects, or Contact.</t>
+          <t>Open studio link / page loads.</t>
         </is>
       </c>
       <c r="H62" s="13" t="inlineStr">
         <is>
-          <t>Navigate to selected route via recovery nav.</t>
+          <t>Protected Defendre Solutions link and nonce-bearing deferred Vercel Insights script.</t>
         </is>
       </c>
       <c r="I62" s="13" t="inlineStr">
         <is>
-          <t>nav aria-label="Page recovery"; two-column mobile grid/row at sm; 48px controls.</t>
+          <t>Focusable external link; nonce sourced from request headers.</t>
         </is>
       </c>
       <c r="J62" s="13" t="inlineStr">
         <is>
-          <t>src/app/not-found.tsx:13-29,70-84</t>
+          <t>src/app/not-found.tsx:31-32,87-103</t>
         </is>
       </c>
       <c r="K62" s="13" t="inlineStr">
         <is>
-          <t>src/app/not-found.test.tsx:27-46</t>
+          <t>src/app/not-found.test.tsx:27-46; proxy nonce coverage is indirect</t>
         </is>
       </c>
       <c r="L62" s="13" t="inlineStr">
@@ -7696,13 +7714,17 @@
       </c>
       <c r="N62" s="13" t="inlineStr">
         <is>
-          <t>Pass — Accessibility tree exposes Page recovery navigation; keyboard Home and click Projects/Contact each reached the intended route; mobile controls reflow 2+1 and remain clear of the dock. Evidence: /tmp/portfolio-feature-audit/baseline/core/not-found-1440-a11y.txt; /tmp/portfolio-feature-audit/baseline/core/not-found-recovery-home-keyboard.txt; /tmp/portfolio-feature-audit/baseline/core/not-found-recovery-projects.txt; /tmp/portfolio-feature-audit/baseline/core/not-found-recovery-contact.txt; /tmp/portfolio-feature-audit/baseline/core/not-found-390-full.png</t>
-        </is>
-      </c>
-      <c r="O62" s="13" t="n"/>
+          <t>Pass — Built by Defendre Solutions is present and opens the correct protected new tab. The analytics script is injected, while existing local-only CAND-RUNTIME-ANALYTICS-001 is confirmed by its 404/MIME console errors; production was not tested. Evidence: /tmp/portfolio-feature-audit/baseline/core/not-found-1440-a11y.txt; /tmp/portfolio-feature-audit/baseline/core/not-found-attribution-studio-tabs.txt; /tmp/portfolio-feature-audit/baseline/core/not-found-analytics-dom.json; /tmp/portfolio-feature-audit/baseline/core/not-found-console.txt; /tmp/portfolio-feature-audit/baseline/core/not-found-network.txt</t>
+        </is>
+      </c>
+      <c r="O62" s="13" t="inlineStr">
+        <is>
+          <t>A11Y-EXT-001; CAND-RUNTIME-ANALYTICS-001</t>
+        </is>
+      </c>
       <c r="P62" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="Q62" s="13" t="inlineStr">
@@ -7712,7 +7734,7 @@
       </c>
       <c r="R62" s="13" t="inlineStr">
         <is>
-          <t>Pass — The labelled recovery navigation rendered three 47.6px+ targets; each was activated and reached its intended route. Evidence: /tmp/portfolio-feature-audit/postfix/core/390/not-found-diagnostics.json; /tmp/portfolio-feature-audit/postfix/core/390/recovery-home-url.txt; /tmp/portfolio-feature-audit/postfix/core/390/recovery-projects-url.txt; /tmp/portfolio-feature-audit/postfix/core/390/recovery-contact-url.txt</t>
+          <t>Pass — The repaired attribution name disclosed its new tab, used protected rel, and opened the studio. The deferred Insights script carried a runtime nonce. Its endpoint is unavailable locally, matching the previously rejected local-only analytics observation rather than a product regression. Evidence: /tmp/portfolio-feature-audit/postfix/core/390/not-found-diagnostics.json; /tmp/portfolio-feature-audit/postfix/core/external/not-found-studio-tabs.txt; /tmp/portfolio-feature-audit/postfix/core/1440/final-console.txt</t>
         </is>
       </c>
       <c r="S62" s="13" t="inlineStr"/>
@@ -7731,7 +7753,7 @@
     <row r="63">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>PF-404-003</t>
+          <t>PF-SEO-001</t>
         </is>
       </c>
       <c r="B63" s="13" t="inlineStr">
@@ -7741,47 +7763,47 @@
       </c>
       <c r="C63" s="13" t="inlineStr">
         <is>
-          <t>Custom not found attribution/analytics</t>
+          <t>Root metadata / all routes</t>
         </is>
       </c>
       <c r="D63" s="13" t="inlineStr">
         <is>
-          <t>Visitor/operator</t>
+          <t>Search/social crawler</t>
         </is>
       </c>
       <c r="E63" s="13" t="inlineStr">
         <is>
-          <t>As a visitor/operator, I want attribution and page-view telemetry.</t>
+          <t>As a crawler, I want canonical site identity and preview cards.</t>
         </is>
       </c>
       <c r="F63" s="13" t="inlineStr">
         <is>
-          <t>404 shown.</t>
+          <t>Metadata rendered.</t>
         </is>
       </c>
       <c r="G63" s="13" t="inlineStr">
         <is>
-          <t>Open studio link / page loads.</t>
+          <t>Parse document head.</t>
         </is>
       </c>
       <c r="H63" s="13" t="inlineStr">
         <is>
-          <t>Protected Defendre Solutions link and nonce-bearing deferred Vercel Insights script.</t>
+          <t>Title/description, canonical URL, Open Graph website fields/image, Twitter large image card.</t>
         </is>
       </c>
       <c r="I63" s="13" t="inlineStr">
         <is>
-          <t>Focusable external link; nonce sourced from request headers.</t>
+          <t>Absolute base normalized from environment; image has dimensions/alt.</t>
         </is>
       </c>
       <c r="J63" s="13" t="inlineStr">
         <is>
-          <t>src/app/not-found.tsx:31-32,87-103</t>
+          <t>src/lib/site-metadata.ts:3-50; src/app/layout.tsx:4-7</t>
         </is>
       </c>
       <c r="K63" s="13" t="inlineStr">
         <is>
-          <t>src/app/not-found.test.tsx:27-46; proxy nonce coverage is indirect</t>
+          <t>src/app/(site)/layout.test.tsx:98-164; src/app/(site)/layout_extended.test.tsx:62-97</t>
         </is>
       </c>
       <c r="L63" s="13" t="inlineStr">
@@ -7796,17 +7818,17 @@
       </c>
       <c r="N63" s="13" t="inlineStr">
         <is>
-          <t>Pass — Built by Defendre Solutions is present and opens the correct protected new tab. The analytics script is injected, while existing local-only CAND-RUNTIME-ANALYTICS-001 is confirmed by its 404/MIME console errors; production was not tested. Evidence: /tmp/portfolio-feature-audit/baseline/core/not-found-1440-a11y.txt; /tmp/portfolio-feature-audit/baseline/core/not-found-attribution-studio-tabs.txt; /tmp/portfolio-feature-audit/baseline/core/not-found-analytics-dom.json; /tmp/portfolio-feature-audit/baseline/core/not-found-console.txt; /tmp/portfolio-feature-audit/baseline/core/not-found-network.txt</t>
+          <t>Pass — Public route metadata used the correct production absolute origin; local fallback divergence was environment-only. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md</t>
         </is>
       </c>
       <c r="O63" s="13" t="inlineStr">
         <is>
-          <t>A11Y-EXT-001; CAND-RUNTIME-ANALYTICS-001</t>
+          <t>CAND-RUNTIME-METADATA-001</t>
         </is>
       </c>
       <c r="P63" s="13" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Won't Fix</t>
         </is>
       </c>
       <c r="Q63" s="13" t="inlineStr">
@@ -7816,7 +7838,7 @@
       </c>
       <c r="R63" s="13" t="inlineStr">
         <is>
-          <t>Pass — The repaired attribution name disclosed its new tab, used protected rel, and opened the studio. The deferred Insights script carried a runtime nonce. Its endpoint is unavailable locally, matching the previously rejected local-only analytics observation rather than a product regression. Evidence: /tmp/portfolio-feature-audit/postfix/core/390/not-found-diagnostics.json; /tmp/portfolio-feature-audit/postfix/core/external/not-found-studio-tabs.txt; /tmp/portfolio-feature-audit/postfix/core/1440/final-console.txt</t>
+          <t>Pass — Root and route-specific title, description, canonical, Open Graph, Twitter/image metadata remained present. Local fallback divergence is environment-only and prior public evidence is green. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/home-static.png; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
         </is>
       </c>
       <c r="S63" s="13" t="inlineStr"/>
@@ -7835,7 +7857,7 @@
     <row r="64">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>PF-SEO-001</t>
+          <t>PF-SEO-002</t>
         </is>
       </c>
       <c r="B64" s="13" t="inlineStr">
@@ -7845,47 +7867,47 @@
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>Root metadata / all routes</t>
+          <t>Metadata URL normalization</t>
         </is>
       </c>
       <c r="D64" s="13" t="inlineStr">
         <is>
-          <t>Search/social crawler</t>
+          <t>Deployment system/crawler</t>
         </is>
       </c>
       <c r="E64" s="13" t="inlineStr">
         <is>
-          <t>As a crawler, I want canonical site identity and preview cards.</t>
+          <t>As a deploy system, I want stable absolute URLs.</t>
         </is>
       </c>
       <c r="F64" s="13" t="inlineStr">
         <is>
-          <t>Metadata rendered.</t>
+          <t>Env vars may be bare, protocol-relative, malformed, or absent.</t>
         </is>
       </c>
       <c r="G64" s="13" t="inlineStr">
         <is>
-          <t>Parse document head.</t>
+          <t>Resolve metadata/robots/sitemap base.</t>
         </is>
       </c>
       <c r="H64" s="13" t="inlineStr">
         <is>
-          <t>Title/description, canonical URL, Open Graph website fields/image, Twitter large image card.</t>
+          <t>Prefer NEXT_PUBLIC_SITE_URL, then production Vercel URL, then deployment URL, then localhost; add https when needed; strip path to root; skip malformed.</t>
         </is>
       </c>
       <c r="I64" s="13" t="inlineStr">
         <is>
-          <t>Absolute base normalized from environment; image has dimensions/alt.</t>
+          <t>Operational, not visual.</t>
         </is>
       </c>
       <c r="J64" s="13" t="inlineStr">
         <is>
-          <t>src/lib/site-metadata.ts:3-50; src/app/layout.tsx:4-7</t>
+          <t>src/lib/site-metadata.ts:3-27; same normalization in src/app/robots.ts:3-30 and src/app/sitemap.ts:3-30</t>
         </is>
       </c>
       <c r="K64" s="13" t="inlineStr">
         <is>
-          <t>src/app/(site)/layout.test.tsx:98-164; src/app/(site)/layout_extended.test.tsx:62-97</t>
+          <t>src/app/(site)/layout.test.tsx:98-151; src/app/(site)/layout_extended.test.tsx:62-97; metadata route tests below</t>
         </is>
       </c>
       <c r="L64" s="13" t="inlineStr">
@@ -7900,7 +7922,7 @@
       </c>
       <c r="N64" s="13" t="inlineStr">
         <is>
-          <t>Pass — Public route metadata used the correct production absolute origin; local fallback divergence was environment-only. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md</t>
+          <t>Pass — Unit suite passed normalization variants and public endpoints consistently used the production origin. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md; /tmp/portfolio-feature-audit/baseline/contact-system/validation-evidence.md</t>
         </is>
       </c>
       <c r="O64" s="13" t="inlineStr">
@@ -7920,7 +7942,7 @@
       </c>
       <c r="R64" s="13" t="inlineStr">
         <is>
-          <t>Pass — Root and route-specific title, description, canonical, Open Graph, Twitter/image metadata remained present. Local fallback divergence is environment-only and prior public evidence is green. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/home-static.png; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
+          <t>Pass — No-env runtime correctly selected localhost fallback; recorded unit/integration coverage validates normalization and precedence variants. Evidence: /tmp/portfolio-feature-audit/postfix/integration-report.md; /tmp/portfolio-feature-audit/postfix/validation-results.json</t>
         </is>
       </c>
       <c r="S64" s="13" t="inlineStr"/>
@@ -7939,7 +7961,7 @@
     <row r="65">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>PF-SEO-002</t>
+          <t>PF-SEO-003</t>
         </is>
       </c>
       <c r="B65" s="13" t="inlineStr">
@@ -7949,47 +7971,47 @@
       </c>
       <c r="C65" s="13" t="inlineStr">
         <is>
-          <t>Metadata URL normalization</t>
+          <t>/robots.txt</t>
         </is>
       </c>
       <c r="D65" s="13" t="inlineStr">
         <is>
-          <t>Deployment system/crawler</t>
+          <t>Search crawler</t>
         </is>
       </c>
       <c r="E65" s="13" t="inlineStr">
         <is>
-          <t>As a deploy system, I want stable absolute URLs.</t>
+          <t>As a crawler, I want crawl instructions.</t>
         </is>
       </c>
       <c r="F65" s="13" t="inlineStr">
         <is>
-          <t>Env vars may be bare, protocol-relative, malformed, or absent.</t>
+          <t>Metadata route requested.</t>
         </is>
       </c>
       <c r="G65" s="13" t="inlineStr">
         <is>
-          <t>Resolve metadata/robots/sitemap base.</t>
+          <t>GET robots.</t>
         </is>
       </c>
       <c r="H65" s="13" t="inlineStr">
         <is>
-          <t>Prefer NEXT_PUBLIC_SITE_URL, then production Vercel URL, then deployment URL, then localhost; add https when needed; strip path to root; skip malformed.</t>
+          <t>Allow all agents at /, emit canonical sitemap URL and host.</t>
         </is>
       </c>
       <c r="I65" s="13" t="inlineStr">
         <is>
-          <t>Operational, not visual.</t>
+          <t>Machine-readable.</t>
         </is>
       </c>
       <c r="J65" s="13" t="inlineStr">
         <is>
-          <t>src/lib/site-metadata.ts:3-27; same normalization in src/app/robots.ts:3-30 and src/app/sitemap.ts:3-30</t>
+          <t>src/app/robots.ts:32-42</t>
         </is>
       </c>
       <c r="K65" s="13" t="inlineStr">
         <is>
-          <t>src/app/(site)/layout.test.tsx:98-151; src/app/(site)/layout_extended.test.tsx:62-97; metadata route tests below</t>
+          <t>src/app/robots.test.ts:42-48</t>
         </is>
       </c>
       <c r="L65" s="13" t="inlineStr">
@@ -8004,7 +8026,7 @@
       </c>
       <c r="N65" s="13" t="inlineStr">
         <is>
-          <t>Pass — Unit suite passed normalization variants and public endpoints consistently used the production origin. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md; /tmp/portfolio-feature-audit/baseline/contact-system/validation-evidence.md</t>
+          <t>Pass — Local endpoint was machine-readable; public robots consistently emitted production Host and Sitemap. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md</t>
         </is>
       </c>
       <c r="O65" s="13" t="inlineStr">
@@ -8024,7 +8046,7 @@
       </c>
       <c r="R65" s="13" t="inlineStr">
         <is>
-          <t>Pass — No-env runtime correctly selected localhost fallback; recorded unit/integration coverage validates normalization and precedence variants. Evidence: /tmp/portfolio-feature-audit/postfix/integration-report.md; /tmp/portfolio-feature-audit/postfix/validation-results.json</t>
+          <t>Pass — Robots returned 200 text/plain with allow-all, host, and sitemap; local values reflect fallback while recorded public values use production. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/robots.png; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
         </is>
       </c>
       <c r="S65" s="13" t="inlineStr"/>
@@ -8043,7 +8065,7 @@
     <row r="66">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>PF-SEO-003</t>
+          <t>PF-SEO-004</t>
         </is>
       </c>
       <c r="B66" s="13" t="inlineStr">
@@ -8053,7 +8075,7 @@
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>/robots.txt</t>
+          <t>/sitemap.xml</t>
         </is>
       </c>
       <c r="D66" s="13" t="inlineStr">
@@ -8063,7 +8085,7 @@
       </c>
       <c r="E66" s="13" t="inlineStr">
         <is>
-          <t>As a crawler, I want crawl instructions.</t>
+          <t>As a crawler, I want core route discovery.</t>
         </is>
       </c>
       <c r="F66" s="13" t="inlineStr">
@@ -8073,27 +8095,27 @@
       </c>
       <c r="G66" s="13" t="inlineStr">
         <is>
-          <t>GET robots.</t>
+          <t>GET sitemap.</t>
         </is>
       </c>
       <c r="H66" s="13" t="inlineStr">
         <is>
-          <t>Allow all agents at /, emit canonical sitemap URL and host.</t>
+          <t>Emit / priority 1, /contact .9, /projects .8, /about .7, all monthly.</t>
         </is>
       </c>
       <c r="I66" s="13" t="inlineStr">
         <is>
-          <t>Machine-readable.</t>
+          <t>Machine-readable; absolute URLs.</t>
         </is>
       </c>
       <c r="J66" s="13" t="inlineStr">
         <is>
-          <t>src/app/robots.ts:32-42</t>
+          <t>src/app/sitemap.ts:32-47</t>
         </is>
       </c>
       <c r="K66" s="13" t="inlineStr">
         <is>
-          <t>src/app/robots.test.ts:42-48</t>
+          <t>src/app/sitemap.test.ts:42-50</t>
         </is>
       </c>
       <c r="L66" s="13" t="inlineStr">
@@ -8108,7 +8130,7 @@
       </c>
       <c r="N66" s="13" t="inlineStr">
         <is>
-          <t>Pass — Local endpoint was machine-readable; public robots consistently emitted production Host and Sitemap. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md</t>
+          <t>Pass — Public sitemap exactly matched all routes, priorities, monthly cadence, and production URLs. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md</t>
         </is>
       </c>
       <c r="O66" s="13" t="inlineStr">
@@ -8128,7 +8150,7 @@
       </c>
       <c r="R66" s="13" t="inlineStr">
         <is>
-          <t>Pass — Robots returned 200 text/plain with allow-all, host, and sitemap; local values reflect fallback while recorded public values use production. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/robots.png; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
+          <t>Pass — Sitemap returned 200 XML with all four routes, monthly cadence, and priorities 1, .8, .7, .9. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/sitemap.png; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
         </is>
       </c>
       <c r="S66" s="13" t="inlineStr"/>
@@ -8147,7 +8169,7 @@
     <row r="67">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>PF-SEO-004</t>
+          <t>PF-OPS-001</t>
         </is>
       </c>
       <c r="B67" s="13" t="inlineStr">
@@ -8157,47 +8179,47 @@
       </c>
       <c r="C67" s="13" t="inlineStr">
         <is>
-          <t>/sitemap.xml</t>
+          <t>Home request pipeline /</t>
         </is>
       </c>
       <c r="D67" s="13" t="inlineStr">
         <is>
-          <t>Search crawler</t>
+          <t>Visitor/deployment system</t>
         </is>
       </c>
       <c r="E67" s="13" t="inlineStr">
         <is>
-          <t>As a crawler, I want core route discovery.</t>
+          <t>As a visitor, I want a fast static home with current content.</t>
         </is>
       </c>
       <c r="F67" s="13" t="inlineStr">
         <is>
-          <t>Metadata route requested.</t>
+          <t>Build has valid committed static assets.</t>
         </is>
       </c>
       <c r="G67" s="13" t="inlineStr">
         <is>
-          <t>GET sitemap.</t>
+          <t>Request /.</t>
         </is>
       </c>
       <c r="H67" s="13" t="inlineStr">
         <is>
-          <t>Emit / priority 1, /contact .9, /projects .8, /about .7, all monthly.</t>
+          <t>Before-files rewrite serves /static-home-internal, whose GET reads the hashed committed HTML; public URL remains /.</t>
         </is>
       </c>
       <c r="I67" s="13" t="inlineStr">
         <is>
-          <t>Machine-readable; absolute URLs.</t>
+          <t>Static document includes semantic/authored home, responsive metadata and one analytics script.</t>
         </is>
       </c>
       <c r="J67" s="13" t="inlineStr">
         <is>
-          <t>src/app/sitemap.ts:32-47</t>
+          <t>next.config.ts:22-25; src/app/static-home-internal/route.ts:3-18; src/generated/static-home-assets.ts:1-7; scripts/render-static-home.tsx:6-19</t>
         </is>
       </c>
       <c r="K67" s="13" t="inlineStr">
         <is>
-          <t>src/app/sitemap.test.ts:42-50</t>
+          <t>src/proxy.test.ts:5-14; src/app/(home)/layout.test.tsx:19-35; static checks in scripts/check-static-home-assets.node-test.mjs:27-46</t>
         </is>
       </c>
       <c r="L67" s="13" t="inlineStr">
@@ -8212,7 +8234,7 @@
       </c>
       <c r="N67" s="13" t="inlineStr">
         <is>
-          <t>Pass — Public sitemap exactly matched all routes, priorities, monthly cadence, and production URLs. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md</t>
+          <t>Pass — Home returned 200 at /, used committed hashed HTML, had one Insights script and zero Next client scripts; static integrity passed. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md; /tmp/portfolio-feature-audit/baseline/contact-system/validation-evidence.md</t>
         </is>
       </c>
       <c r="O67" s="13" t="inlineStr">
@@ -8232,7 +8254,7 @@
       </c>
       <c r="R67" s="13" t="inlineStr">
         <is>
-          <t>Pass — Sitemap returned 200 XML with all four routes, monthly cadence, and priorities 1, .8, .7, .9. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/sitemap.png; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
+          <t>Pass — Home served current committed static HTML with one Insights script, zero Next client chunks, expected metadata and content. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/home-static.png; /tmp/portfolio-feature-audit/postfix/contact-system/lane-c-trace.zip</t>
         </is>
       </c>
       <c r="S67" s="13" t="inlineStr"/>
@@ -8251,7 +8273,7 @@
     <row r="68">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>PF-OPS-001</t>
+          <t>PF-OPS-002</t>
         </is>
       </c>
       <c r="B68" s="13" t="inlineStr">
@@ -8261,47 +8283,47 @@
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>Home request pipeline /</t>
+          <t>Static home cache/security</t>
         </is>
       </c>
       <c r="D68" s="13" t="inlineStr">
         <is>
-          <t>Visitor/deployment system</t>
+          <t>Browser/CDN</t>
         </is>
       </c>
       <c r="E68" s="13" t="inlineStr">
         <is>
-          <t>As a visitor, I want a fast static home with current content.</t>
+          <t>As a browser/CDN, I want immutable assets and secure HTML.</t>
         </is>
       </c>
       <c r="F68" s="13" t="inlineStr">
         <is>
-          <t>Build has valid committed static assets.</t>
+          <t>Hashed static home files exist.</t>
         </is>
       </c>
       <c r="G68" s="13" t="inlineStr">
         <is>
-          <t>Request /.</t>
+          <t>Request home/static asset.</t>
         </is>
       </c>
       <c r="H68" s="13" t="inlineStr">
         <is>
-          <t>Before-files rewrite serves /static-home-internal, whose GET reads the hashed committed HTML; public URL remains /.</t>
+          <t>HTML gets year-long shared cache + 1-day SWR and strict CSP/security headers; hashed HTML/CSS get immutable one-year cache.</t>
         </is>
       </c>
       <c r="I68" s="13" t="inlineStr">
         <is>
-          <t>Static document includes semantic/authored home, responsive metadata and one analytics script.</t>
+          <t>Machine-level policy; static CSP allows only self/blob/data as declared and blocks framing.</t>
         </is>
       </c>
       <c r="J68" s="13" t="inlineStr">
         <is>
-          <t>next.config.ts:22-25; src/app/static-home-internal/route.ts:3-18; src/generated/static-home-assets.ts:1-7; scripts/render-static-home.tsx:6-19</t>
+          <t>src/app/static-home-internal/route.ts:7-17; next.config.ts:26-40</t>
         </is>
       </c>
       <c r="K68" s="13" t="inlineStr">
         <is>
-          <t>src/proxy.test.ts:5-14; src/app/(home)/layout.test.tsx:19-35; static checks in scripts/check-static-home-assets.node-test.mjs:27-46</t>
+          <t>scripts/check-static-home-runtime.mjs:4-13; no direct header integration test</t>
         </is>
       </c>
       <c r="L68" s="13" t="inlineStr">
@@ -8316,17 +8338,13 @@
       </c>
       <c r="N68" s="13" t="inlineStr">
         <is>
-          <t>Pass — Home returned 200 at /, used committed hashed HTML, had one Insights script and zero Next client scripts; static integrity passed. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md; /tmp/portfolio-feature-audit/baseline/contact-system/validation-evidence.md</t>
-        </is>
-      </c>
-      <c r="O68" s="13" t="inlineStr">
-        <is>
-          <t>CAND-RUNTIME-METADATA-001</t>
-        </is>
-      </c>
+          <t>Pass — Home cache and CSP matched; hashed HTML/CSS privacy/cache behavior passed. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md</t>
+        </is>
+      </c>
+      <c r="O68" s="13" t="n"/>
       <c r="P68" s="13" t="inlineStr">
         <is>
-          <t>Won't Fix</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="Q68" s="13" t="inlineStr">
@@ -8336,7 +8354,7 @@
       </c>
       <c r="R68" s="13" t="inlineStr">
         <is>
-          <t>Pass — Home served current committed static HTML with one Insights script, zero Next client chunks, expected metadata and content. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/home-static.png; /tmp/portfolio-feature-audit/postfix/contact-system/lane-c-trace.zip</t>
+          <t>Pass — Home shared cache/SWR, static CSP/security headers, and immutable content-addressed CSS cache matched expectations. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system-report.md</t>
         </is>
       </c>
       <c r="S68" s="13" t="inlineStr"/>
@@ -8355,7 +8373,7 @@
     <row r="69">
       <c r="A69" s="13" t="inlineStr">
         <is>
-          <t>PF-OPS-002</t>
+          <t>PF-OPS-003</t>
         </is>
       </c>
       <c r="B69" s="13" t="inlineStr">
@@ -8365,47 +8383,47 @@
       </c>
       <c r="C69" s="13" t="inlineStr">
         <is>
-          <t>Static home cache/security</t>
+          <t>Static implementation URL privacy</t>
         </is>
       </c>
       <c r="D69" s="13" t="inlineStr">
         <is>
-          <t>Browser/CDN</t>
+          <t>Visitor/crawler</t>
         </is>
       </c>
       <c r="E69" s="13" t="inlineStr">
         <is>
-          <t>As a browser/CDN, I want immutable assets and secure HTML.</t>
+          <t>As a visitor/crawler, I should not browse implementation URLs.</t>
         </is>
       </c>
       <c r="F69" s="13" t="inlineStr">
         <is>
-          <t>Hashed static home files exist.</t>
+          <t>Request /static-home-internal or hashed static-home HTML directly.</t>
         </is>
       </c>
       <c r="G69" s="13" t="inlineStr">
         <is>
-          <t>Request home/static asset.</t>
+          <t>GET implementation path.</t>
         </is>
       </c>
       <c r="H69" s="13" t="inlineStr">
         <is>
-          <t>HTML gets year-long shared cache + 1-day SWR and strict CSP/security headers; hashed HTML/CSS get immutable one-year cache.</t>
+          <t>308 redirect to /; matcher excludes framework/API assets as configured.</t>
         </is>
       </c>
       <c r="I69" s="13" t="inlineStr">
         <is>
-          <t>Machine-level policy; static CSP allows only self/blob/data as declared and blocks framing.</t>
+          <t>Keeps crawlable surface canonical.</t>
         </is>
       </c>
       <c r="J69" s="13" t="inlineStr">
         <is>
-          <t>src/app/static-home-internal/route.ts:7-17; next.config.ts:26-40</t>
+          <t>src/proxy.ts:7-16,52-61</t>
         </is>
       </c>
       <c r="K69" s="13" t="inlineStr">
         <is>
-          <t>scripts/check-static-home-runtime.mjs:4-13; no direct header integration test</t>
+          <t>src/proxy.test.ts:5-14</t>
         </is>
       </c>
       <c r="L69" s="13" t="inlineStr">
@@ -8420,7 +8438,7 @@
       </c>
       <c r="N69" s="13" t="inlineStr">
         <is>
-          <t>Pass — Home cache and CSP matched; hashed HTML/CSS privacy/cache behavior passed. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md</t>
+          <t>Pass — Both internal and hashed HTML paths returned 308 with Location /. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md</t>
         </is>
       </c>
       <c r="O69" s="13" t="n"/>
@@ -8436,7 +8454,7 @@
       </c>
       <c r="R69" s="13" t="inlineStr">
         <is>
-          <t>Pass — Home shared cache/SWR, static CSP/security headers, and immutable content-addressed CSS cache matched expectations. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system-report.md</t>
+          <t>Pass — Internal and current hashed static-home HTML implementation paths each returned 308 Location /. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system-report.md</t>
         </is>
       </c>
       <c r="S69" s="13" t="inlineStr"/>
@@ -8455,7 +8473,7 @@
     <row r="70">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>PF-OPS-003</t>
+          <t>PF-OPS-004</t>
         </is>
       </c>
       <c r="B70" s="13" t="inlineStr">
@@ -8465,47 +8483,47 @@
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>Static implementation URL privacy</t>
+          <t>Dynamic route CSP nonce</t>
         </is>
       </c>
       <c r="D70" s="13" t="inlineStr">
         <is>
-          <t>Visitor/crawler</t>
+          <t>Browser/security system</t>
         </is>
       </c>
       <c r="E70" s="13" t="inlineStr">
         <is>
-          <t>As a visitor/crawler, I should not browse implementation URLs.</t>
+          <t>As a browser, I want scripts constrained by per-request CSP.</t>
         </is>
       </c>
       <c r="F70" s="13" t="inlineStr">
         <is>
-          <t>Request /static-home-internal or hashed static-home HTML directly.</t>
+          <t>Request non-home matched route.</t>
         </is>
       </c>
       <c r="G70" s="13" t="inlineStr">
         <is>
-          <t>GET implementation path.</t>
+          <t>Load page.</t>
         </is>
       </c>
       <c r="H70" s="13" t="inlineStr">
         <is>
-          <t>308 redirect to /; matcher excludes framework/API assets as configured.</t>
+          <t>Generate nonce, attach to request headers and response CSP; scripts require self + nonce + strict-dynamic; local dev alone permits unsafe-eval; images allow Microlink.</t>
         </is>
       </c>
       <c r="I70" s="13" t="inlineStr">
         <is>
-          <t>Keeps crawlable surface canonical.</t>
+          <t>Blocks objects/framing and restricts base/form; local HTTP omits upgrade directive.</t>
         </is>
       </c>
       <c r="J70" s="13" t="inlineStr">
         <is>
-          <t>src/proxy.ts:7-16,52-61</t>
+          <t>src/proxy.ts:18-49</t>
         </is>
       </c>
       <c r="K70" s="13" t="inlineStr">
         <is>
-          <t>src/proxy.test.ts:5-14</t>
+          <t>src/proxy.test.ts:15-35</t>
         </is>
       </c>
       <c r="L70" s="13" t="inlineStr">
@@ -8520,13 +8538,17 @@
       </c>
       <c r="N70" s="13" t="inlineStr">
         <is>
-          <t>Pass — Both internal and hashed HTML paths returned 308 with Location /. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md</t>
-        </is>
-      </c>
-      <c r="O70" s="13" t="n"/>
+          <t>Pass — All 21 body nonces matched the response nonce; directives and local HTTP behavior matched. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md</t>
+        </is>
+      </c>
+      <c r="O70" s="13" t="inlineStr">
+        <is>
+          <t>PERF-NAV-001</t>
+        </is>
+      </c>
       <c r="P70" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Won't Fix</t>
         </is>
       </c>
       <c r="Q70" s="13" t="inlineStr">
@@ -8536,7 +8558,7 @@
       </c>
       <c r="R70" s="13" t="inlineStr">
         <is>
-          <t>Pass — Internal and current hashed static-home HTML implementation paths each returned 308 Location /. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system-report.md</t>
+          <t>Pass — Dynamic route response used a per-response nonce CSP with strict script policy; recorded integration verified all body nonce matches. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/lane-c-trace.zip; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
         </is>
       </c>
       <c r="S70" s="13" t="inlineStr"/>
@@ -8555,7 +8577,7 @@
     <row r="71">
       <c r="A71" s="13" t="inlineStr">
         <is>
-          <t>PF-OPS-004</t>
+          <t>PF-OPS-005</t>
         </is>
       </c>
       <c r="B71" s="13" t="inlineStr">
@@ -8565,7 +8587,7 @@
       </c>
       <c r="C71" s="13" t="inlineStr">
         <is>
-          <t>Dynamic route CSP nonce</t>
+          <t>Site-wide security headers</t>
         </is>
       </c>
       <c r="D71" s="13" t="inlineStr">
@@ -8575,37 +8597,37 @@
       </c>
       <c r="E71" s="13" t="inlineStr">
         <is>
-          <t>As a browser, I want scripts constrained by per-request CSP.</t>
+          <t>As a visitor, I want hardened responses.</t>
         </is>
       </c>
       <c r="F71" s="13" t="inlineStr">
         <is>
-          <t>Request non-home matched route.</t>
+          <t>Any path matches Next headers.</t>
         </is>
       </c>
       <c r="G71" s="13" t="inlineStr">
         <is>
-          <t>Load page.</t>
+          <t>Load response.</t>
         </is>
       </c>
       <c r="H71" s="13" t="inlineStr">
         <is>
-          <t>Generate nonce, attach to request headers and response CSP; scripts require self + nonce + strict-dynamic; local dev alone permits unsafe-eval; images allow Microlink.</t>
+          <t>Disable camera/geolocation/microphone/payment; strict-origin referrer; two-year HSTS; nosniff.</t>
         </is>
       </c>
       <c r="I71" s="13" t="inlineStr">
         <is>
-          <t>Blocks objects/framing and restricts base/form; local HTTP omits upgrade directive.</t>
+          <t>Operational security.</t>
         </is>
       </c>
       <c r="J71" s="13" t="inlineStr">
         <is>
-          <t>src/proxy.ts:18-49</t>
+          <t>next.config.ts:3-20,36-40; mirrored on static HTML src/app/static-home-internal/route.ts:12-16</t>
         </is>
       </c>
       <c r="K71" s="13" t="inlineStr">
         <is>
-          <t>src/proxy.test.ts:15-35</t>
+          <t>No direct integration test; CSP-focused unit tests only</t>
         </is>
       </c>
       <c r="L71" s="13" t="inlineStr">
@@ -8620,17 +8642,13 @@
       </c>
       <c r="N71" s="13" t="inlineStr">
         <is>
-          <t>Pass — All 21 body nonces matched the response nonce; directives and local HTTP behavior matched. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md</t>
-        </is>
-      </c>
-      <c r="O71" s="13" t="inlineStr">
-        <is>
-          <t>PERF-NAV-001</t>
-        </is>
-      </c>
+          <t>Pass — All four header families matched locally and publicly. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md</t>
+        </is>
+      </c>
+      <c r="O71" s="13" t="n"/>
       <c r="P71" s="13" t="inlineStr">
         <is>
-          <t>Won't Fix</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="Q71" s="13" t="inlineStr">
@@ -8640,7 +8658,7 @@
       </c>
       <c r="R71" s="13" t="inlineStr">
         <is>
-          <t>Pass — Dynamic route response used a per-response nonce CSP with strict script policy; recorded integration verified all body nonce matches. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/lane-c-trace.zip; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
+          <t>Pass — Expected Permissions, Referrer, HSTS, and nosniff headers appeared across Home, dynamic, metadata, and asset responses. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system-report.md</t>
         </is>
       </c>
       <c r="S71" s="13" t="inlineStr"/>
@@ -8659,7 +8677,7 @@
     <row r="72">
       <c r="A72" s="13" t="inlineStr">
         <is>
-          <t>PF-OPS-005</t>
+          <t>PF-OPS-006</t>
         </is>
       </c>
       <c r="B72" s="13" t="inlineStr">
@@ -8669,47 +8687,47 @@
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>Site-wide security headers</t>
+          <t>Analytics loading</t>
         </is>
       </c>
       <c r="D72" s="13" t="inlineStr">
         <is>
-          <t>Browser/security system</t>
+          <t>Site operator</t>
         </is>
       </c>
       <c r="E72" s="13" t="inlineStr">
         <is>
-          <t>As a visitor, I want hardened responses.</t>
+          <t>As an operator, I want page analytics on all route shells.</t>
         </is>
       </c>
       <c r="F72" s="13" t="inlineStr">
         <is>
-          <t>Any path matches Next headers.</t>
+          <t>Browser loads a route.</t>
         </is>
       </c>
       <c r="G72" s="13" t="inlineStr">
         <is>
-          <t>Load response.</t>
+          <t>Page rendered.</t>
         </is>
       </c>
       <c r="H72" s="13" t="inlineStr">
         <is>
-          <t>Disable camera/geolocation/microphone/payment; strict-origin referrer; two-year HSTS; nosniff.</t>
+          <t>Home/404 load deferred same-origin Insights script (nonce where dynamic); site routes mount Vercel Analytics React adapter.</t>
         </is>
       </c>
       <c r="I72" s="13" t="inlineStr">
         <is>
-          <t>Operational security.</t>
+          <t>Analytics failure does not block primary behaviors; home avoids Next client chunks.</t>
         </is>
       </c>
       <c r="J72" s="13" t="inlineStr">
         <is>
-          <t>next.config.ts:3-20,36-40; mirrored on static HTML src/app/static-home-internal/route.ts:12-16</t>
+          <t>src/app/(home)/layout.tsx:4-11; src/app/(site)/layout.tsx:2,53-54; src/app/not-found.tsx:31-32,102; scripts/render-static-home.tsx:18</t>
         </is>
       </c>
       <c r="K72" s="13" t="inlineStr">
         <is>
-          <t>No direct integration test; CSP-focused unit tests only</t>
+          <t>src/app/(home)/layout.test.tsx:19-35; src/app/(site)/layout.test.tsx:152-164; scripts/check-static-home-runtime.mjs:12</t>
         </is>
       </c>
       <c r="L72" s="13" t="inlineStr">
@@ -8724,13 +8742,17 @@
       </c>
       <c r="N72" s="13" t="inlineStr">
         <is>
-          <t>Pass — All four header families matched locally and publicly. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md</t>
-        </is>
-      </c>
-      <c r="O72" s="13" t="n"/>
+          <t>Pass — Public Insights script returned 200 JavaScript; site Analytics emitted Contact event; local static script 404 remained nonblocking and environment-only. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md</t>
+        </is>
+      </c>
+      <c r="O72" s="13" t="inlineStr">
+        <is>
+          <t>CAND-RUNTIME-ANALYTICS-001</t>
+        </is>
+      </c>
       <c r="P72" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Won't Fix</t>
         </is>
       </c>
       <c r="Q72" s="13" t="inlineStr">
@@ -8740,7 +8762,7 @@
       </c>
       <c r="R72" s="13" t="inlineStr">
         <is>
-          <t>Pass — Expected Permissions, Referrer, HSTS, and nosniff headers appeared across Home, dynamic, metadata, and asset responses. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system-report.md</t>
+          <t>Pass — Home retained one Insights loader and Contact emitted the expected minimal custom event. Local Insights script 404 is a known nonblocking hosting limitation; recorded public delivery is 200 JavaScript. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/lane-c-trace.zip; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
         </is>
       </c>
       <c r="S72" s="13" t="inlineStr"/>
@@ -8759,7 +8781,7 @@
     <row r="73">
       <c r="A73" s="13" t="inlineStr">
         <is>
-          <t>PF-OPS-006</t>
+          <t>PF-OPS-007</t>
         </is>
       </c>
       <c r="B73" s="13" t="inlineStr">
@@ -8769,47 +8791,47 @@
       </c>
       <c r="C73" s="13" t="inlineStr">
         <is>
-          <t>Analytics loading</t>
+          <t>Responsive image delivery</t>
         </is>
       </c>
       <c r="D73" s="13" t="inlineStr">
         <is>
-          <t>Site operator</t>
+          <t>Browser</t>
         </is>
       </c>
       <c r="E73" s="13" t="inlineStr">
         <is>
-          <t>As an operator, I want page analytics on all route shells.</t>
+          <t>As a visitor, I want appropriately sized local images.</t>
         </is>
       </c>
       <c r="F73" s="13" t="inlineStr">
         <is>
-          <t>Browser loads a route.</t>
+          <t>Next image optimizer available.</t>
         </is>
       </c>
       <c r="G73" s="13" t="inlineStr">
         <is>
-          <t>Page rendered.</t>
+          <t>Load headshot/project preview.</t>
         </is>
       </c>
       <c r="H73" s="13" t="inlineStr">
         <is>
-          <t>Home/404 load deferred same-origin Insights script (nonce where dynamic); site routes mount Vercel Analytics React adapter.</t>
+          <t>Emit optimizer URLs for 256-3840 widths, srcSet, authored sizes, async decoding, eager/high priority for priority images and lazy otherwise.</t>
         </is>
       </c>
       <c r="I73" s="13" t="inlineStr">
         <is>
-          <t>Analytics failure does not block primary behaviors; home avoids Next client chunks.</t>
+          <t>Descriptive alt required by component contract; reduces bandwidth across sizes.</t>
         </is>
       </c>
       <c r="J73" s="13" t="inlineStr">
         <is>
-          <t>src/app/(home)/layout.tsx:4-11; src/app/(site)/layout.tsx:2,53-54; src/app/not-found.tsx:31-32,102; scripts/render-static-home.tsx:18</t>
+          <t>src/components/ResponsiveImage.tsx:1-43; remote Microlink pattern next.config.ts:42-49</t>
         </is>
       </c>
       <c r="K73" s="13" t="inlineStr">
         <is>
-          <t>src/app/(home)/layout.test.tsx:19-35; src/app/(site)/layout.test.tsx:152-164; scripts/check-static-home-runtime.mjs:12</t>
+          <t>Project image behavior src/components/__tests__/ProjectCard.test.tsx:79-93,151-159; no width-selection browser assertion</t>
         </is>
       </c>
       <c r="L73" s="13" t="inlineStr">
@@ -8824,17 +8846,17 @@
       </c>
       <c r="N73" s="13" t="inlineStr">
         <is>
-          <t>Pass — Public Insights script returned 200 JavaScript; site Analytics emitted Contact event; local static script 404 remained nonblocking and environment-only. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md</t>
+          <t>Pass — Markup and HTTP assets matched; unnecessary hidden/below-fold preloads confirm an existing performance candidate but not delivery failure. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system/home-mobile-loading.png; /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md</t>
         </is>
       </c>
       <c r="O73" s="13" t="inlineStr">
         <is>
-          <t>CAND-RUNTIME-ANALYTICS-001</t>
+          <t>PERF-IMG-001</t>
         </is>
       </c>
       <c r="P73" s="13" t="inlineStr">
         <is>
-          <t>Won't Fix</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="Q73" s="13" t="inlineStr">
@@ -8844,7 +8866,7 @@
       </c>
       <c r="R73" s="13" t="inlineStr">
         <is>
-          <t>Pass — Home retained one Insights loader and Contact emitted the expected minimal custom event. Local Insights script 404 is a known nonblocking hosting limitation; recorded public delivery is 200 JavaScript. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/lane-c-trace.zip; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
+          <t>Pass — Responsive optimizer markup and image priorities were correct; hero alone eager/high, navigation/project imagery lazy/non-high; asset requests succeeded. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/home-static.png; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
         </is>
       </c>
       <c r="S73" s="13" t="inlineStr"/>
@@ -8863,7 +8885,7 @@
     <row r="74">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>PF-OPS-007</t>
+          <t>PF-OPS-008</t>
         </is>
       </c>
       <c r="B74" s="13" t="inlineStr">
@@ -8873,47 +8895,47 @@
       </c>
       <c r="C74" s="13" t="inlineStr">
         <is>
-          <t>Responsive image delivery</t>
+          <t>Static home integrity pipeline</t>
         </is>
       </c>
       <c r="D74" s="13" t="inlineStr">
         <is>
-          <t>Browser</t>
+          <t>Developer/CI</t>
         </is>
       </c>
       <c r="E74" s="13" t="inlineStr">
         <is>
-          <t>As a visitor, I want appropriately sized local images.</t>
+          <t>As a maintainer, I want stale committed home output rejected.</t>
         </is>
       </c>
       <c r="F74" s="13" t="inlineStr">
         <is>
-          <t>Next image optimizer available.</t>
+          <t>Run build/check scripts.</t>
         </is>
       </c>
       <c r="G74" s="13" t="inlineStr">
         <is>
-          <t>Load headshot/project preview.</t>
+          <t>npm run prebuild, build, check:static-home, or sync.</t>
         </is>
       </c>
       <c r="H74" s="13" t="inlineStr">
         <is>
-          <t>Emit optimizer URLs for 256-3840 widths, srcSet, authored sizes, async decoding, eager/high priority for priority images and lazy otherwise.</t>
+          <t>Hash explicit source/assets/fonts; compile/minify CSS; server-render HTML; commit manifest; fail when inputs/outputs/cross-links/fonts/runtime invariants drift.</t>
         </is>
       </c>
       <c r="I74" s="13" t="inlineStr">
         <is>
-          <t>Descriptive alt required by component contract; reduces bandwidth across sizes.</t>
+          <t>Build-time behavior; generated home must have zero Next chunks and exactly one Insights script.</t>
         </is>
       </c>
       <c r="J74" s="13" t="inlineStr">
         <is>
-          <t>src/components/ResponsiveImage.tsx:1-43; remote Microlink pattern next.config.ts:42-49</t>
+          <t>package.json:5-15; scripts/static-home-assets-lib.mjs:6-82; scripts/sync-static-home-assets.mjs:10-36; scripts/check-static-home-assets.mjs:5-19; scripts/check-static-home-runtime.mjs:4-13</t>
         </is>
       </c>
       <c r="K74" s="13" t="inlineStr">
         <is>
-          <t>Project image behavior src/components/__tests__/ProjectCard.test.tsx:79-93,151-159; no width-selection browser assertion</t>
+          <t>scripts/check-static-home-assets.node-test.mjs:27-46</t>
         </is>
       </c>
       <c r="L74" s="13" t="inlineStr">
@@ -8928,17 +8950,17 @@
       </c>
       <c r="N74" s="13" t="inlineStr">
         <is>
-          <t>Pass — Markup and HTTP assets matched; unnecessary hidden/below-fold preloads confirm an existing performance candidate but not delivery failure. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system/home-mobile-loading.png; /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md</t>
+          <t>Pass — Prebuild, build runtime check, static tests, and check:static-home all passed with hash 209f3c04064b013e. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/validation-evidence.md</t>
         </is>
       </c>
       <c r="O74" s="13" t="inlineStr">
         <is>
-          <t>PERF-IMG-001</t>
+          <t>CAND-RUNTIME-METADATA-001</t>
         </is>
       </c>
       <c r="P74" s="13" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Won't Fix</t>
         </is>
       </c>
       <c r="Q74" s="13" t="inlineStr">
@@ -8948,7 +8970,7 @@
       </c>
       <c r="R74" s="13" t="inlineStr">
         <is>
-          <t>Pass — Responsive optimizer markup and image priorities were correct; hero alone eager/high, navigation/project imagery lazy/non-high; asset requests succeeded. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/home-static.png; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
+          <t>Pass — Current static-home asset/runtime check passed with input hash prefix 9210fbac0dc0b3bb; recorded clean build also passed. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system-report.md; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
         </is>
       </c>
       <c r="S74" s="13" t="inlineStr"/>
@@ -8967,7 +8989,7 @@
     <row r="75">
       <c r="A75" s="13" t="inlineStr">
         <is>
-          <t>PF-OPS-008</t>
+          <t>PF-OPS-009</t>
         </is>
       </c>
       <c r="B75" s="13" t="inlineStr">
@@ -8977,47 +8999,47 @@
       </c>
       <c r="C75" s="13" t="inlineStr">
         <is>
-          <t>Static home integrity pipeline</t>
+          <t>Self-hosted static fonts</t>
         </is>
       </c>
       <c r="D75" s="13" t="inlineStr">
         <is>
-          <t>Developer/CI</t>
+          <t>Browser/build system</t>
         </is>
       </c>
       <c r="E75" s="13" t="inlineStr">
         <is>
-          <t>As a maintainer, I want stale committed home output rejected.</t>
+          <t>As a visitor, I want stable typography without third-party font requests.</t>
         </is>
       </c>
       <c r="F75" s="13" t="inlineStr">
         <is>
-          <t>Run build/check scripts.</t>
+          <t>Static font files present and hashes valid.</t>
         </is>
       </c>
       <c r="G75" s="13" t="inlineStr">
         <is>
-          <t>npm run prebuild, build, check:static-home, or sync.</t>
+          <t>Load static home.</t>
         </is>
       </c>
       <c r="H75" s="13" t="inlineStr">
         <is>
-          <t>Hash explicit source/assets/fonts; compile/minify CSS; server-render HTML; commit manifest; fail when inputs/outputs/cross-links/fonts/runtime invariants drift.</t>
+          <t>Serve Fraunces/Manrope WOFF2 subsets with font-display: swap and metric-compatible fallbacks; reject missing/tampered fonts.</t>
         </is>
       </c>
       <c r="I75" s="13" t="inlineStr">
         <is>
-          <t>Build-time behavior; generated home must have zero Next chunks and exactly one Insights script.</t>
+          <t>Covers Latin/extended, Vietnamese, Cyrillic, Greek subsets as configured; avoids invisible text.</t>
         </is>
       </c>
       <c r="J75" s="13" t="inlineStr">
         <is>
-          <t>package.json:5-15; scripts/static-home-assets-lib.mjs:6-82; scripts/sync-static-home-assets.mjs:10-36; scripts/check-static-home-assets.mjs:5-19; scripts/check-static-home-runtime.mjs:4-13</t>
+          <t>scripts/static-home-fonts.mjs:5-34; public/static-home/fonts/*; src/lib/fonts.ts:1-13</t>
         </is>
       </c>
       <c r="K75" s="13" t="inlineStr">
         <is>
-          <t>scripts/check-static-home-assets.node-test.mjs:27-46</t>
+          <t>Integrity covered by scripts/check-static-home-assets.node-test.mjs:27-46; no visual font test</t>
         </is>
       </c>
       <c r="L75" s="13" t="inlineStr">
@@ -9032,17 +9054,13 @@
       </c>
       <c r="N75" s="13" t="inlineStr">
         <is>
-          <t>Pass — Prebuild, build runtime check, static tests, and check:static-home all passed with hash 209f3c04064b013e. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/validation-evidence.md</t>
-        </is>
-      </c>
-      <c r="O75" s="13" t="inlineStr">
-        <is>
-          <t>CAND-RUNTIME-METADATA-001</t>
-        </is>
-      </c>
+          <t>Pass — All authored font files and CSS declarations were present; static integrity passed. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md; /tmp/portfolio-feature-audit/baseline/contact-system/validation-evidence.md</t>
+        </is>
+      </c>
+      <c r="O75" s="13" t="n"/>
       <c r="P75" s="13" t="inlineStr">
         <is>
-          <t>Won't Fix</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="Q75" s="13" t="inlineStr">
@@ -9052,7 +9070,7 @@
       </c>
       <c r="R75" s="13" t="inlineStr">
         <is>
-          <t>Pass — Current static-home asset/runtime check passed with input hash prefix 9210fbac0dc0b3bb; recorded clean build also passed. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system-report.md; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
+          <t>Pass — Self-hosted Fraunces/Manrope CSS and font-display swap remained; integrity check validated font hashes. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/home-static.png; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
         </is>
       </c>
       <c r="S75" s="13" t="inlineStr"/>
@@ -9071,7 +9089,7 @@
     <row r="76">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>PF-OPS-009</t>
+          <t>PF-OPS-010</t>
         </is>
       </c>
       <c r="B76" s="13" t="inlineStr">
@@ -9081,47 +9099,47 @@
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>Self-hosted static fonts</t>
+          <t>Automated quality gates</t>
         </is>
       </c>
       <c r="D76" s="13" t="inlineStr">
         <is>
-          <t>Browser/build system</t>
+          <t>Developer/CI</t>
         </is>
       </c>
       <c r="E76" s="13" t="inlineStr">
         <is>
-          <t>As a visitor, I want stable typography without third-party font requests.</t>
+          <t>As a maintainer, I want repeatable validation.</t>
         </is>
       </c>
       <c r="F76" s="13" t="inlineStr">
         <is>
-          <t>Static font files present and hashes valid.</t>
+          <t>Dependencies installed.</t>
         </is>
       </c>
       <c r="G76" s="13" t="inlineStr">
         <is>
-          <t>Load static home.</t>
+          <t>Run scripts.</t>
         </is>
       </c>
       <c r="H76" s="13" t="inlineStr">
         <is>
-          <t>Serve Fraunces/Manrope WOFF2 subsets with font-display: swap and metric-compatible fallbacks; reject missing/tampered fonts.</t>
+          <t>lint ESLint; test Vitest/jsdom max 2 workers excluding E2E; test:e2e Playwright Chromium one worker with failure artifacts; build Next + static runtime check.</t>
         </is>
       </c>
       <c r="I76" s="13" t="inlineStr">
         <is>
-          <t>Covers Latin/extended, Vietnamese, Cyrillic, Greek subsets as configured; avoids invisible text.</t>
+          <t>E2E explicitly covers mobile 390, tablet 768, desktop 1440 nav; contact mobile; projects desktop.</t>
         </is>
       </c>
       <c r="J76" s="13" t="inlineStr">
         <is>
-          <t>scripts/static-home-fonts.mjs:5-34; public/static-home/fonts/*; src/lib/fonts.ts:1-13</t>
+          <t>package.json:5-15; vitest.config.ts:5-18; playwright.config.ts:9-43; playwright.config.helpers.ts:1-8</t>
         </is>
       </c>
       <c r="K76" s="13" t="inlineStr">
         <is>
-          <t>Integrity covered by scripts/check-static-home-assets.node-test.mjs:27-46; no visual font test</t>
+          <t>Config classifier playwright.config.test.ts:5-13; E2E specs e2e/*.spec.ts</t>
         </is>
       </c>
       <c r="L76" s="13" t="inlineStr">
@@ -9136,13 +9154,17 @@
       </c>
       <c r="N76" s="13" t="inlineStr">
         <is>
-          <t>Pass — All authored font files and CSS declarations were present; static integrity passed. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md; /tmp/portfolio-feature-audit/baseline/contact-system/validation-evidence.md</t>
-        </is>
-      </c>
-      <c r="O76" s="13" t="n"/>
+          <t>Pass — 145 unit, 2 static, and 6 E2E tests passed; lint passed with one existing warning; clean tsc and build passed. Cross-engine/mode coverage remains a confirmed QA candidate. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/validation-evidence.md</t>
+        </is>
+      </c>
+      <c r="O76" s="13" t="inlineStr">
+        <is>
+          <t>QA-A11Y-001</t>
+        </is>
+      </c>
       <c r="P76" s="13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="Q76" s="13" t="inlineStr">
@@ -9152,7 +9174,7 @@
       </c>
       <c r="R76" s="13" t="inlineStr">
         <is>
-          <t>Pass — Self-hosted Fraunces/Manrope CSS and font-display swap remained; integrity check validated font hashes. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/home-static.png; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
+          <t>Pass — Recorded final gates: 156/156 unit, 3/3 static, typecheck/build/static integrity, and 18/18 browser tests across Chromium/Firefox/WebKit. Current config includes the three browser projects and focused accessibility spec. Evidence: /tmp/portfolio-feature-audit/postfix/integration-report.md; /tmp/portfolio-feature-audit/postfix/validation-results.json</t>
         </is>
       </c>
       <c r="S76" s="13" t="inlineStr"/>
@@ -9171,7 +9193,7 @@
     <row r="77">
       <c r="A77" s="13" t="inlineStr">
         <is>
-          <t>PF-OPS-010</t>
+          <t>PF-OPS-011</t>
         </is>
       </c>
       <c r="B77" s="13" t="inlineStr">
@@ -9181,47 +9203,47 @@
       </c>
       <c r="C77" s="13" t="inlineStr">
         <is>
-          <t>Automated quality gates</t>
+          <t>Public asset catalog</t>
         </is>
       </c>
       <c r="D77" s="13" t="inlineStr">
         <is>
-          <t>Developer/CI</t>
+          <t>Browser</t>
         </is>
       </c>
       <c r="E77" s="13" t="inlineStr">
         <is>
-          <t>As a maintainer, I want repeatable validation.</t>
+          <t>As a visitor, I want the authored media used by the portfolio.</t>
         </is>
       </c>
       <c r="F77" s="13" t="inlineStr">
         <is>
-          <t>Dependencies installed.</t>
+          <t>Asset request.</t>
         </is>
       </c>
       <c r="G77" s="13" t="inlineStr">
         <is>
-          <t>Run scripts.</t>
+          <t>Load icon/headshot/project preview.</t>
         </is>
       </c>
       <c r="H77" s="13" t="inlineStr">
         <is>
-          <t>lint ESLint; test Vitest/jsdom max 2 workers excluding E2E; test:e2e Playwright Chromium one worker with failure artifacts; build Next + static runtime check.</t>
+          <t>Serve favicon, headshot, and seven project-preview JPGs; static-home HTML/CSS/fonts are content-addressed.</t>
         </is>
       </c>
       <c r="I77" s="13" t="inlineStr">
         <is>
-          <t>E2E explicitly covers mobile 390, tablet 768, desktop 1440 nav; contact mobile; projects desktop.</t>
+          <t>Image components provide alt except decorative fallbacks; favicon linked by static renderer.</t>
         </is>
       </c>
       <c r="J77" s="13" t="inlineStr">
         <is>
-          <t>package.json:5-15; vitest.config.ts:5-18; playwright.config.ts:9-43; playwright.config.helpers.ts:1-8</t>
+          <t>public/favicon via src/app/favicon.ico; public/headshot.jpg; public/project-previews/*; scripts/render-static-home.tsx:17; catalog references src/data/projects.ts:24-87</t>
         </is>
       </c>
       <c r="K77" s="13" t="inlineStr">
         <is>
-          <t>Config classifier playwright.config.test.ts:5-13; E2E specs e2e/*.spec.ts</t>
+          <t>Project catalog required fields/assets partly covered by src/data/__tests__/projects.test.ts:14-134; no file-existence unit test outside static hash pipeline</t>
         </is>
       </c>
       <c r="L77" s="13" t="inlineStr">
@@ -9236,17 +9258,13 @@
       </c>
       <c r="N77" s="13" t="inlineStr">
         <is>
-          <t>Pass — 145 unit, 2 static, and 6 E2E tests passed; lint passed with one existing warning; clean tsc and build passed. Cross-engine/mode coverage remains a confirmed QA candidate. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/validation-evidence.md</t>
-        </is>
-      </c>
-      <c r="O77" s="13" t="inlineStr">
-        <is>
-          <t>QA-A11Y-001</t>
-        </is>
-      </c>
+          <t>Pass — All nine asset requests returned 200 with correct MIME and nonzero bytes; content-addressed artifacts verified. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md</t>
+        </is>
+      </c>
+      <c r="O77" s="13" t="n"/>
       <c r="P77" s="13" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="Q77" s="13" t="inlineStr">
@@ -9256,7 +9274,7 @@
       </c>
       <c r="R77" s="13" t="inlineStr">
         <is>
-          <t>Pass — Recorded final gates: 156/156 unit, 3/3 static, typecheck/build/static integrity, and 18/18 browser tests across Chromium/Firefox/WebKit. Current config includes the three browser projects and focused accessibility spec. Evidence: /tmp/portfolio-feature-audit/postfix/integration-report.md; /tmp/portfolio-feature-audit/postfix/validation-results.json</t>
+          <t>Pass — Favicon, headshot, and seven project preview files returned 9/9 HTTP 200 with correct MIME and nonzero bytes. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system-report.md</t>
         </is>
       </c>
       <c r="S77" s="13" t="inlineStr"/>
@@ -9275,7 +9293,7 @@
     <row r="78">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>PF-OPS-011</t>
+          <t>PF-OPS-012</t>
         </is>
       </c>
       <c r="B78" s="13" t="inlineStr">
@@ -9285,52 +9303,52 @@
       </c>
       <c r="C78" s="13" t="inlineStr">
         <is>
-          <t>Public asset catalog</t>
+          <t>Dormant Three.js subsystem</t>
         </is>
       </c>
       <c r="D78" s="13" t="inlineStr">
         <is>
-          <t>Browser</t>
+          <t>Maintainer (not current visitor)</t>
         </is>
       </c>
       <c r="E78" s="13" t="inlineStr">
         <is>
-          <t>As a visitor, I want the authored media used by the portfolio.</t>
+          <t>As a maintainer, I want legacy WebGL code identified accurately.</t>
         </is>
       </c>
       <c r="F78" s="13" t="inlineStr">
         <is>
-          <t>Asset request.</t>
+          <t>ThreeScene is imported/mounted (it currently is not; AnimatedBackground deliberately replaced it).</t>
         </is>
       </c>
       <c r="G78" s="13" t="inlineStr">
         <is>
-          <t>Load icon/headshot/project preview.</t>
+          <t>Mount component.</t>
         </is>
       </c>
       <c r="H78" s="13" t="inlineStr">
         <is>
-          <t>Serve favicon, headshot, and seven project-preview JPGs; static-home HTML/CSS/fonts are content-addressed.</t>
+          <t>Would create a pointer-reactive Three.js scene, pause/resume per interactivity state, debounce resize, cap DPR/delta, render a static gradient if setup fails, and dispose resources. Current production shell renders CSS ambient background instead.</t>
         </is>
       </c>
       <c r="I78" s="13" t="inlineStr">
         <is>
-          <t>Image components provide alt except decorative fallbacks; favicon linked by static renderer.</t>
+          <t>Container is pointer-events none; failure keeps fallback; motion lifecycle tested. Not an active user-visible feature.</t>
         </is>
       </c>
       <c r="J78" s="13" t="inlineStr">
         <is>
-          <t>public/favicon via src/app/favicon.ico; public/headshot.jpg; public/project-previews/*; scripts/render-static-home.tsx:17; catalog references src/data/projects.ts:24-87</t>
+          <t>src/components/ThreeScene.tsx:1-22; src/hooks/three/useThreeScene.ts:8-64; src/hooks/three/useThreeBase.ts:8-79; src/hooks/three/useThreeAnimation.ts:18-116; active replacement src/components/AnimatedBackground.tsx:1-14</t>
         </is>
       </c>
       <c r="K78" s="13" t="inlineStr">
         <is>
-          <t>Project catalog required fields/assets partly covered by src/data/__tests__/projects.test.ts:14-134; no file-existence unit test outside static hash pipeline</t>
+          <t>src/components/__tests__/AnimatedBackground.test.tsx:17-24; src/components/__tests__/ThreeScene*.test.tsx; src/hooks/three/__tests__/*.test.ts</t>
         </is>
       </c>
       <c r="L78" s="13" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Inactive / Dormant</t>
         </is>
       </c>
       <c r="M78" s="13" t="inlineStr">
@@ -9340,7 +9358,7 @@
       </c>
       <c r="N78" s="13" t="inlineStr">
         <is>
-          <t>Pass — All nine asset requests returned 200 with correct MIME and nonzero bytes; content-addressed artifacts verified. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md</t>
+          <t>Pass — No active production import/mount exists; lifecycle/failure/performance tests passed in the unit suite. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md; /tmp/portfolio-feature-audit/baseline/contact-system/validation-evidence.md</t>
         </is>
       </c>
       <c r="O78" s="13" t="n"/>
@@ -9356,10 +9374,14 @@
       </c>
       <c r="R78" s="13" t="inlineStr">
         <is>
-          <t>Pass — Favicon, headshot, and seven project preview files returned 9/9 HTTP 200 with correct MIME and nonzero bytes. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system-report.md</t>
-        </is>
-      </c>
-      <c r="S78" s="13" t="inlineStr"/>
+          <t>Pass — Active Home had AnimatedBackground and zero canvas/Three.js mounts; recorded unit/integration coverage validates dormant lifecycle and cleanup. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/home-static.png; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
+        </is>
+      </c>
+      <c r="S78" s="13" t="inlineStr">
+        <is>
+          <t>Dormant, unmounted Three.js subsystem retained for code-inventory completeness.</t>
+        </is>
+      </c>
       <c r="T78" s="13" t="inlineStr">
         <is>
           <t>Unassigned</t>
@@ -9372,112 +9394,8 @@
         <v>46257.6050925926</v>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="13" t="inlineStr">
-        <is>
-          <t>PF-OPS-012</t>
-        </is>
-      </c>
-      <c r="B79" s="13" t="inlineStr">
-        <is>
-          <t>Code Inventory</t>
-        </is>
-      </c>
-      <c r="C79" s="13" t="inlineStr">
-        <is>
-          <t>Dormant Three.js subsystem</t>
-        </is>
-      </c>
-      <c r="D79" s="13" t="inlineStr">
-        <is>
-          <t>Maintainer (not current visitor)</t>
-        </is>
-      </c>
-      <c r="E79" s="13" t="inlineStr">
-        <is>
-          <t>As a maintainer, I want legacy WebGL code identified accurately.</t>
-        </is>
-      </c>
-      <c r="F79" s="13" t="inlineStr">
-        <is>
-          <t>ThreeScene is imported/mounted (it currently is not; AnimatedBackground deliberately replaced it).</t>
-        </is>
-      </c>
-      <c r="G79" s="13" t="inlineStr">
-        <is>
-          <t>Mount component.</t>
-        </is>
-      </c>
-      <c r="H79" s="13" t="inlineStr">
-        <is>
-          <t>Would create a pointer-reactive Three.js scene, pause/resume per interactivity state, debounce resize, cap DPR/delta, render a static gradient if setup fails, and dispose resources. Current production shell renders CSS ambient background instead.</t>
-        </is>
-      </c>
-      <c r="I79" s="13" t="inlineStr">
-        <is>
-          <t>Container is pointer-events none; failure keeps fallback; motion lifecycle tested. Not an active user-visible feature.</t>
-        </is>
-      </c>
-      <c r="J79" s="13" t="inlineStr">
-        <is>
-          <t>src/components/ThreeScene.tsx:1-22; src/hooks/three/useThreeScene.ts:8-64; src/hooks/three/useThreeBase.ts:8-79; src/hooks/three/useThreeAnimation.ts:18-116; active replacement src/components/AnimatedBackground.tsx:1-14</t>
-        </is>
-      </c>
-      <c r="K79" s="13" t="inlineStr">
-        <is>
-          <t>src/components/__tests__/AnimatedBackground.test.tsx:17-24; src/components/__tests__/ThreeScene*.test.tsx; src/hooks/three/__tests__/*.test.ts</t>
-        </is>
-      </c>
-      <c r="L79" s="13" t="inlineStr">
-        <is>
-          <t>Inactive / Dormant</t>
-        </is>
-      </c>
-      <c r="M79" s="13" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="N79" s="13" t="inlineStr">
-        <is>
-          <t>Pass — No active production import/mount exists; lifecycle/failure/performance tests passed in the unit suite. Evidence: /tmp/portfolio-feature-audit/baseline/contact-system/system-evidence.md; /tmp/portfolio-feature-audit/baseline/contact-system/validation-evidence.md</t>
-        </is>
-      </c>
-      <c r="O79" s="13" t="n"/>
-      <c r="P79" s="13" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="Q79" s="13" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="R79" s="13" t="inlineStr">
-        <is>
-          <t>Pass — Active Home had AnimatedBackground and zero canvas/Three.js mounts; recorded unit/integration coverage validates dormant lifecycle and cleanup. Evidence: /tmp/portfolio-feature-audit/postfix/contact-system/home-static.png; /tmp/portfolio-feature-audit/postfix/integration-report.md</t>
-        </is>
-      </c>
-      <c r="S79" s="13" t="inlineStr">
-        <is>
-          <t>Dormant, unmounted Three.js subsystem retained for code-inventory completeness.</t>
-        </is>
-      </c>
-      <c r="T79" s="13" t="inlineStr">
-        <is>
-          <t>Unassigned</t>
-        </is>
-      </c>
-      <c r="U79" s="18" t="n">
-        <v>46257</v>
-      </c>
-      <c r="V79" s="18" t="n">
-        <v>46257.6050925926</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:V79"/>
+  <autoFilter ref="A1:V78"/>
   <conditionalFormatting sqref="M2:M79">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>M2="Not Run"</formula>

</xml_diff>